<commit_message>
incorporated latest CDEL & ILAO feedback
</commit_message>
<xml_diff>
--- a/docassemble/PowerOfAttorneyHealthCare/data/sources/poa_hc_es.xlsx
+++ b/docassemble/PowerOfAttorneyHealthCare/data/sources/poa_hc_es.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{702F067C-3D08-41ED-868D-E66DFCC589C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60905B48-AB5B-4C17-86EE-127EA6AE26FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-34770" yWindow="-4050" windowWidth="32145" windowHeight="17925" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -11041,32 +11041,6 @@
     <t>Testigo</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Este programa no ofrece asesoramiento legal. No sustituye al asesoramiento de un abogado.
-El uso de este programa no crea una relación abogado-cliente entre usted e Illinois Legal Aid Online ni sus empleados.
-Los videos en este programa ofrecen información importante sobre el proceso de planificación anticipada. Proporcionan únicamente información, no asesoramiento legal. No crean una relación abogado-cliente entre usted y el Center for Disability and Elder Law ni sus empleados.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ collapse_template(get_legal_help) }</t>
-    </r>
-  </si>
-  <si>
     <t>Otorgante</t>
   </si>
   <si>
@@ -11169,94 +11143,6 @@
     <t>**¿Qué pasa si he cambiado legalmente mi nombre?**</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if for_yourself == True:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">¿Eres residente de Illinois?
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% else:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>¿</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">${principal.name_full()} </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri (Body)"/>
-      </rPr>
-      <t xml:space="preserve">es </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">residente de Illinois?
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>% endif</t>
-    </r>
-  </si>
-  <si>
     <t>Lo sentimos</t>
   </si>
   <si>
@@ -11448,224 +11334,6 @@
         <scheme val="minor"/>
       </rPr>
       <t>% endif</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${collapse_template(video_who_agent)}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if for_yourself == False:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">El agente es la persona en quien </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${principal.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> confía para tomar decisiones sobre su atención médica. Es muy importante que </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF2967FA"/>
-        <rFont val="Calibri (Body)"/>
-      </rPr>
-      <t>${principal.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0096FF"/>
-        <rFont val="Calibri (Body)"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">hable con su agente sobre sus deseos y sentimientos con respecto a la atención médica, incluidas las decisiones al final de la vida. Las conversaciones significativas guiarán el juicio del agente y asegurarán que ambos estén de acuerdo.
-Un agente tiene mucho poder, y es posible que pueda abusar de ese poder. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${principal.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> debe elegir a alguien en quien confíe con su salud y bienestar.
-El agente es la persona que tomará decisiones médicas por </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${principal.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> si </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${principal.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> está demasiado enfermo(a) para tomar o comunicar sus propias decisiones.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% else:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Tu agente es la persona en quien confías para tomar decisiones sobre tu atención médica por ti. Es muy importante hablar con tu agente sobre tus deseos y sentimientos con respecto a la atención médica, incluidas las decisiones al final de la vida. Las conversaciones significativas contigo guiarán su juicio y asegurarán que ambos estén de acuerdo.
-Un agente tiene mucho poder, y es posible que pueda abusar de ese poder. Debes elegir a alguien en quien confíes para tu salud y bienestar.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif  
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${collapse_template(agent_require)}</t>
     </r>
   </si>
   <si>
@@ -13097,35 +12765,6 @@
   </si>
   <si>
     <t>Acerca de poner fin a un Poder Notarial</t>
-  </si>
-  <si>
-    <t>Tengo una preferencia específica. (Explica abajo)</t>
-  </si>
-  <si>
-    <t>Tiene una preferencia específica. (Explica abajo)</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${subject_do_does}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> no autorizan que se suspendan ciertos tratamientos. (Explica abajo)</t>
-    </r>
   </si>
   <si>
     <t>Capacidad legal</t>
@@ -16157,172 +15796,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">"Nominar" significa sugerir o proponer a una persona que un tribunal puede elegir para actuar como tutor legal.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if for_yourself == True:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Un tribunal puede considerar necesario nombrar a un tutor legal para administrar tu salud y bienestar. Un tutor puede tomar decisiones sobre asuntos aparte de la atención médica y, por lo general, tendría derechos, poderes y responsabilidades sobre ti similares a los que tienen los padres sobre sus hijos menores. 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% else:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Un tribunal puede considerar necesario designar a un tutor legal para administrar la salud y el bienestar de </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${principal.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. Un tutor puede tomar decisiones sobre asuntos aparte de la atención médica y, por lo general, tendría derechos, poderes y responsabilidades sobre </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${principal.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> similares a los que tienen los padres sobre sus hijos menores.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Si haces clic en **No**, entonces un tribunal puede nombrar a alguien distinto de </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${agent.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> como tutor si es necesario. Incluso si haces clic en **Sí**, un tribunal aún podría nombrar a otra persona como tutor si determina que </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${agent.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> está incumpliendo con sus deberes</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
       <t xml:space="preserve">Este Poder Notarial entrará en vigor cuando </t>
     </r>
     <r>
@@ -17174,29 +16647,6 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> no autorizo una autopsia. (on behalf of principal) no autoriza una autopsia.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${subject_do_does}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> (for self) no autorizo/ no autoriza que se inicien ciertos tratamientos. (Explica abajo)</t>
     </r>
   </si>
   <si>
@@ -18499,68 +17949,6 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> a la ciencia.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Para usar este programa necesitarás saber:
-* El nombre, la ciudad, el estado y el número de teléfono de alguien en quien confías para tomar decisiones sobre tu atención médica por ti y que será tu **{agente}**, y
-* El nombre, la ciudad, el estado y el número de teléfono de cualquier **{agentes sucesores}**.
-El programa te preguntará:
-* Cuándo quieres que tu agente comience a tomar decisiones, y
-* Qué quieres que tu agente haga con respecto a tu atención médica.
-Reserva entre 10 y 15 minutos para completar este programa, y más tiempo si ves los videos. Puedes iniciar sesión y guardar tu progreso para regresar más tarde. 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ collapse_template(help_example) }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">  
-Haz clic en las **{palabras verdes}** para aprender qué significan. Algunas preguntas tienen un signo de interrogación en un círculo </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ fa_icon("question-circle", color_css="#0DCAF0" ) }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> que también brinda ayuda.</t>
     </r>
   </si>
   <si>
@@ -22427,70 +21815,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if get_language() == 'en':
-:globe: English | [Español](${ interview_url(new_session=1, lang="es") })
-% else:
-:globe: [English](${ interview_url(new_session=1, lang="en") }) | Español
-% endif
-Bienvenido(a) al Formulario Guiado de Poder Notarial para el Cuidado de la Salud de Illinois Legal Aid Online.
-Este programa te ayuda a crear documentos que le otorgan a una persona de tu confianza la autoridad legal para tomar decisiones sobre tu atención médica. Esto significa que esa persona podrá tomar decisiones sobre tu atención médica cuando no puedas hacerlo por ti mismo(a). Si así lo deseas, también puedes autorizarla para que tome decisiones sobre tu atención médica antesde que eso ocurra.
-Este programa incluye videos con información sobre cómo hacer un Poder Notarial para el Cuidado de la Salud. No tienes que verlos, pero pueden serte útiles.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">[YOUTUBE ccToVpEse7s]
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Para obtener más información, lee el artículo de ILAO sobre los [**Conceptos Básicos del Poder Notarial para el Cuidado de la Salud**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://es.illinoislegalaid.org/legal-information/setting-power-attorney-healthcare</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>).</t>
-    </r>
-  </si>
-  <si>
     <t>0f7bfeab41a01c4696b50fcc79df32b5</t>
   </si>
   <si>
@@ -22797,9 +22121,6 @@
       <t xml:space="preserve">'s address below.
 </t>
     </r>
-  </si>
-  <si>
-    <t>Ingrese la dirección de ${agent.name_full()} a continuación.</t>
   </si>
   <si>
     <t>9aa7634ed326cf05a8e3f53a8f59fc2b</t>
@@ -23631,6 +22952,614 @@
       </rPr>
       <t>% endif</t>
     </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if get_language() == 'en':
+:globe: English | [Español](${ interview_url(new_session=1, lang="es") })
+% else:
+:globe: [English](${ interview_url(new_session=1, lang="en") }) | Español
+% endif
+Bienvenido(a) al Formulario Guiado de Poder Notarial para el Cuidado de la Salud de Illinois Legal Aid Online.
+Este programa te ayuda a crear documentos que le otorgan a una persona de tu confianza la autoridad legal para tomar decisiones sobre tu atención médica. Esto significa que esa persona podrá tomar decisiones sobre tu atención médica cuando no puedas hacerlo por ti mismo(a). Si así lo deseas, también puedes autorizarla para que tome decisiones sobre tu atención médica antes de que eso ocurra.
+Este programa incluye videos con información sobre cómo hacer un Poder Notarial para el Cuidado de la Salud. No tienes que verlos, pero pueden serte útiles.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">[YOUTUBE ccToVpEse7s]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Para obtener más información, lee el artículo de ILAO sobre los [**Conceptos Básicos del Poder Notarial para el Cuidado de la Salud**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://es.illinoislegalaid.org/legal-information/setting-power-attorney-healthcare</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Este programa no ofrece asesoramiento legal. No sustituye al asesoramiento de un abogado.
+El uso de este programa no crea una relación abogado-cliente entre ti e Illinois Legal Aid Online ni sus empleados.
+Los videos en este programa ofrecen información importante sobre el proceso de planificación anticipada. Proporcionan únicamente información, no asesoramiento legal. No crean una relación abogado-cliente entre ti y el Center for Disability and Elder Law ni sus empleados.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ collapse_template(get_legal_help) }</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Para usar este programa necesitarás saber:
+* El nombre, la ciudad, el estado y el número de teléfono de alguien en quien confías para tomar decisiones sobre tu atención médica por ti y que será tu **{agente}**, y
+* El nombre, la ciudad, el estado y el número de teléfono de “de los **{agentes sucesores}** que quieras nombrar.
+El programa te preguntará:
+* Cuándo quieres que tu agente comience a tomar decisiones, y
+* Qué quieres que tu agente haga con respecto a tu atención médica.
+Reserva entre 10 y 15 minutos para completar este programa, y más tiempo si ves los videos. Puedes iniciar sesión y guardar tu progreso para regresar más tarde. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ collapse_template(help_example) }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  
+Haz clic en las **{palabras verdes}** para aprender qué significan. Algunas preguntas tienen un signo de interrogación en un círculo </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ fa_icon("question-circle", color_css="#0DCAF0" ) }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> que también brinda ayuda.</t>
+    </r>
+  </si>
+  <si>
+    <t>% if for_yourself == True:
+¿Vives en Illinois?
+% else:
+¿${principal.name_full()} vive en Illinois?
+% endif</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${collapse_template(video_who_agent)}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if for_yourself == False:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">El agente es la persona en quien </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> confía para tomar decisiones sobre su atención médica. Es muy importante que </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF2967FA"/>
+        <rFont val="Calibri (Body)"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0096FF"/>
+        <rFont val="Calibri (Body)"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">hable con su agente sobre sus deseos y sentimientos con respecto a la atención médica, incluidas las decisiones al final de la vida. Tener conversaciones significativas con tu agente ayudará a guiar su juicio y a asegurar que ambos estén de acuerdo.
+Un agente tiene mucho poder, y es posible que pueda abusar de ese poder. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> debe elegir a alguien en quien confíe con su salud y bienestar.
+El agente es la persona que tomará decisiones médicas por </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> si </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> está demasiado enfermo(a) para tomar o comunicar sus propias decisiones.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% else:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Tu agente es la persona en quien confías para tomar decisiones sobre tu atención médica por ti. Es muy importante hablar con tu agente sobre tus deseos y sentimientos con respecto a la atención médica, incluidas las decisiones al final de la vida. Las conversaciones significativas contigo guiarán su juicio y asegurarán que ambos estén de acuerdo.
+Un agente tiene mucho poder, y es posible que pueda abusar de ese poder. Debes elegir a alguien en quien confíes para tu salud y bienestar.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif  
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${collapse_template(agent_require)}</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"Nominar" significa sugerir o proponer a una persona que un tribunal puede elegir para actuar como tutor legal.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if for_yourself == True:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Un tribunal puede considerar necesario nombrar a un tutor legal para administrar tu salud y bienestar. Un tutor puede tomar decisiones sobre asuntos aparte de la atención médica y, por lo general, tendría derechos, poderes y responsabilidades sobre ti similares a los que tienen los padres sobre sus hijos menores. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% else:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Un tribunal puede considerar necesario designar a un tutor legal para administrar la salud y el bienestar de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Un tutor puede tomar decisiones sobre asuntos aparte de la atención médica y, por lo general, tendría derechos, poderes y responsabilidades sobre </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> similares a los que tienen los padres sobre sus hijos menores.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Si haces clic en **No**, entonces un tribunal puede nombrar a alguien distinto de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${agent.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> como tutor si es necesario. Incluso si haces clic en **Sí**, un tribunal aún podría nombrar a otra persona como tutor si determina que </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${agent.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> está incumpliendo con sus deberes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Tengo una preferencia específica. (Explícala abajo)</t>
+  </si>
+  <si>
+    <t>Tiene una preferencia específica. (Explícala abajo)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${subject_do_does}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (for self) no autorizo/ no autoriza que se inicien ciertos tratamientos. (Explícala abajo)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${subject_do_does}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> no autorizan que se suspendan ciertos tratamientos. (Explícala abajo)</t>
+    </r>
+  </si>
+  <si>
+    <t>Ingresa la dirección de ${agent.name_full()} a continuación.</t>
   </si>
 </sst>
 </file>
@@ -23756,7 +23685,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -23781,6 +23710,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -24169,7 +24101,7 @@
         <v>1</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>774</v>
+        <v>765</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>11</v>
@@ -24178,10 +24110,10 @@
         <v>12</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>775</v>
+        <v>766</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>776</v>
+        <v>796</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -24233,7 +24165,7 @@
         <v>20</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -24337,7 +24269,7 @@
         <v>31</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>724</v>
+        <v>798</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="28.8">
@@ -24351,7 +24283,7 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>729</v>
+        <v>720</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>11</v>
@@ -24360,7 +24292,7 @@
         <v>12</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>732</v>
+        <v>723</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>33</v>
@@ -24377,7 +24309,7 @@
         <v>1</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>730</v>
+        <v>721</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>11</v>
@@ -24386,7 +24318,7 @@
         <v>12</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>731</v>
+        <v>722</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>34</v>
@@ -24403,7 +24335,7 @@
         <v>0</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>783</v>
+        <v>773</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>11</v>
@@ -24412,10 +24344,10 @@
         <v>12</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>784</v>
+        <v>774</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>787</v>
+        <v>777</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="216">
@@ -24429,7 +24361,7 @@
         <v>1</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>785</v>
+        <v>775</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>11</v>
@@ -24438,10 +24370,10 @@
         <v>12</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>786</v>
+        <v>776</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>788</v>
+        <v>778</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="28.8">
@@ -24493,7 +24425,7 @@
         <v>41</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>747</v>
+        <v>738</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="28.8">
@@ -24545,21 +24477,21 @@
         <v>47</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>735</v>
+        <v>726</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="115.2">
       <c r="A18" s="2" t="s">
-        <v>742</v>
+        <v>733</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>748</v>
+        <v>739</v>
       </c>
       <c r="C18" s="2">
         <v>0</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>749</v>
+        <v>740</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>11</v>
@@ -24568,18 +24500,18 @@
         <v>12</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>750</v>
+        <v>741</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>751</v>
+        <v>742</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="28.8">
       <c r="A19" s="2" t="s">
-        <v>742</v>
+        <v>733</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>748</v>
+        <v>739</v>
       </c>
       <c r="C19" s="2">
         <v>1</v>
@@ -24623,7 +24555,7 @@
         <v>53</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>576</v>
+        <v>797</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -24649,7 +24581,7 @@
         <v>56</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="43.2">
@@ -24675,7 +24607,7 @@
         <v>58</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>725</v>
+        <v>716</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="57.6">
@@ -24701,7 +24633,7 @@
         <v>60</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>726</v>
+        <v>717</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="28.8">
@@ -24727,7 +24659,7 @@
         <v>62</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="57.6">
@@ -24753,12 +24685,12 @@
         <v>64</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26" s="2" t="s">
-        <v>742</v>
+        <v>733</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>54</v>
@@ -24767,7 +24699,7 @@
         <v>5</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>777</v>
+        <v>767</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>11</v>
@@ -24776,15 +24708,15 @@
         <v>12</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>778</v>
+        <v>768</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>781</v>
+        <v>771</v>
       </c>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="2" t="s">
-        <v>742</v>
+        <v>733</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>54</v>
@@ -24793,7 +24725,7 @@
         <v>6</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>779</v>
+        <v>769</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>11</v>
@@ -24802,10 +24734,10 @@
         <v>12</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>780</v>
+        <v>770</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>782</v>
+        <v>772</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="28.8">
@@ -24831,7 +24763,7 @@
         <v>67</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="244.8">
@@ -24857,7 +24789,7 @@
         <v>69</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="86.4">
@@ -24883,7 +24815,7 @@
         <v>72</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="409.6">
@@ -24897,7 +24829,7 @@
         <v>1</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>759</v>
+        <v>750</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>11</v>
@@ -24906,10 +24838,10 @@
         <v>12</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>760</v>
+        <v>751</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>761</v>
+        <v>752</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -24935,7 +24867,7 @@
         <v>74</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -24961,7 +24893,7 @@
         <v>76</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -24987,7 +24919,7 @@
         <v>78</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -25013,7 +24945,7 @@
         <v>80</v>
       </c>
       <c r="H35" s="8" t="s">
-        <v>756</v>
+        <v>747</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -25065,7 +24997,7 @@
         <v>85</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="100.8">
@@ -25091,7 +25023,7 @@
         <v>88</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="28.8">
@@ -25117,7 +25049,7 @@
         <v>90</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="86.4">
@@ -25142,8 +25074,8 @@
       <c r="G40" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="H40" s="3" t="s">
-        <v>590</v>
+      <c r="H40" s="10" t="s">
+        <v>799</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="28.8">
@@ -25169,7 +25101,7 @@
         <v>96</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="144">
@@ -25195,7 +25127,7 @@
         <v>98</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="86.4">
@@ -25247,7 +25179,7 @@
         <v>105</v>
       </c>
       <c r="H44" s="3" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="374.4">
@@ -25273,7 +25205,7 @@
         <v>107</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>594</v>
+        <v>800</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="86.4">
@@ -25299,7 +25231,7 @@
         <v>110</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="28.8">
@@ -25325,7 +25257,7 @@
         <v>112</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="28.8">
@@ -25351,7 +25283,7 @@
         <v>115</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>697</v>
+        <v>691</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -25377,7 +25309,7 @@
         <v>117</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="43.2">
@@ -25403,12 +25335,12 @@
         <v>119</v>
       </c>
       <c r="H50" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="28.8">
       <c r="A51" s="2" t="s">
-        <v>742</v>
+        <v>733</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>113</v>
@@ -25417,7 +25349,7 @@
         <v>4</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>792</v>
+        <v>782</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>11</v>
@@ -25426,10 +25358,10 @@
         <v>12</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>793</v>
+        <v>783</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>794</v>
+        <v>806</v>
       </c>
     </row>
     <row r="52" spans="1:8">
@@ -25455,7 +25387,7 @@
         <v>121</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
     </row>
     <row r="53" spans="1:8">
@@ -25481,7 +25413,7 @@
         <v>123</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
     </row>
     <row r="54" spans="1:8" ht="129.6">
@@ -25495,7 +25427,7 @@
         <v>0</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>789</v>
+        <v>779</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>11</v>
@@ -25504,10 +25436,10 @@
         <v>12</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>790</v>
+        <v>780</v>
       </c>
       <c r="H54" s="3" t="s">
-        <v>791</v>
+        <v>781</v>
       </c>
     </row>
     <row r="55" spans="1:8" ht="28.8">
@@ -25533,7 +25465,7 @@
         <v>126</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>727</v>
+        <v>718</v>
       </c>
     </row>
     <row r="56" spans="1:8" ht="28.8">
@@ -25585,7 +25517,7 @@
         <v>132</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
     </row>
     <row r="58" spans="1:8" ht="100.8">
@@ -25611,7 +25543,7 @@
         <v>135</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>762</v>
+        <v>753</v>
       </c>
     </row>
     <row r="59" spans="1:8" ht="288">
@@ -25637,7 +25569,7 @@
         <v>137</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>698</v>
+        <v>801</v>
       </c>
     </row>
     <row r="60" spans="1:8" ht="28.8">
@@ -25663,7 +25595,7 @@
         <v>140</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
     </row>
     <row r="61" spans="1:8">
@@ -25715,7 +25647,7 @@
         <v>146</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
     </row>
     <row r="63" spans="1:8" ht="28.8">
@@ -25741,7 +25673,7 @@
         <v>148</v>
       </c>
       <c r="H63" s="3" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
     </row>
     <row r="64" spans="1:8" ht="144">
@@ -25767,7 +25699,7 @@
         <v>150</v>
       </c>
       <c r="H64" s="3" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
     </row>
     <row r="65" spans="1:8">
@@ -25845,7 +25777,7 @@
         <v>158</v>
       </c>
       <c r="H67" s="6" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
     </row>
     <row r="68" spans="1:8" ht="43.2">
@@ -25871,7 +25803,7 @@
         <v>160</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
     </row>
     <row r="69" spans="1:8" ht="57.6">
@@ -25897,7 +25829,7 @@
         <v>162</v>
       </c>
       <c r="H69" s="6" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
     </row>
     <row r="70" spans="1:8">
@@ -25949,7 +25881,7 @@
         <v>168</v>
       </c>
       <c r="H71" s="3" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
     </row>
     <row r="72" spans="1:8" ht="172.8">
@@ -25975,7 +25907,7 @@
         <v>170</v>
       </c>
       <c r="H72" s="3" t="s">
-        <v>699</v>
+        <v>692</v>
       </c>
     </row>
     <row r="73" spans="1:8" ht="28.8">
@@ -26001,7 +25933,7 @@
         <v>172</v>
       </c>
       <c r="H73" s="9" t="s">
-        <v>700</v>
+        <v>693</v>
       </c>
     </row>
     <row r="74" spans="1:8">
@@ -26027,7 +25959,7 @@
         <v>174</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="43.2">
@@ -26053,7 +25985,7 @@
         <v>176</v>
       </c>
       <c r="H75" s="3" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
     </row>
     <row r="76" spans="1:8" ht="57.6">
@@ -26079,7 +26011,7 @@
         <v>178</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>702</v>
+        <v>695</v>
       </c>
     </row>
     <row r="77" spans="1:8">
@@ -26105,7 +26037,7 @@
         <v>180</v>
       </c>
       <c r="H77" s="3" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
     </row>
     <row r="78" spans="1:8" ht="28.8">
@@ -26157,7 +26089,7 @@
         <v>186</v>
       </c>
       <c r="H79" s="3" t="s">
-        <v>701</v>
+        <v>694</v>
       </c>
     </row>
     <row r="80" spans="1:8" ht="115.2">
@@ -26183,7 +26115,7 @@
         <v>189</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
     </row>
     <row r="81" spans="1:8" ht="360">
@@ -26209,7 +26141,7 @@
         <v>191</v>
       </c>
       <c r="H81" s="3" t="s">
-        <v>703</v>
+        <v>696</v>
       </c>
     </row>
     <row r="82" spans="1:8" ht="28.8">
@@ -26235,7 +26167,7 @@
         <v>194</v>
       </c>
       <c r="H82" s="6" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="83" spans="1:8" ht="28.8">
@@ -26258,10 +26190,10 @@
         <v>12</v>
       </c>
       <c r="G83" s="3" t="s">
-        <v>757</v>
+        <v>748</v>
       </c>
       <c r="H83" s="3" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
     </row>
     <row r="84" spans="1:8" ht="72">
@@ -26287,7 +26219,7 @@
         <v>198</v>
       </c>
       <c r="H84" s="3" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
     </row>
     <row r="85" spans="1:8" ht="72">
@@ -26313,7 +26245,7 @@
         <v>200</v>
       </c>
       <c r="H85" s="3" t="s">
-        <v>704</v>
+        <v>697</v>
       </c>
     </row>
     <row r="86" spans="1:8">
@@ -26365,7 +26297,7 @@
         <v>205</v>
       </c>
       <c r="H87" s="3" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
     </row>
     <row r="88" spans="1:8">
@@ -26391,7 +26323,7 @@
         <v>207</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>619</v>
+        <v>616</v>
       </c>
     </row>
     <row r="89" spans="1:8">
@@ -26443,7 +26375,7 @@
         <v>213</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>705</v>
+        <v>698</v>
       </c>
     </row>
     <row r="91" spans="1:8" ht="43.2">
@@ -26469,7 +26401,7 @@
         <v>215</v>
       </c>
       <c r="H91" s="6" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
     </row>
     <row r="92" spans="1:8" ht="43.2">
@@ -26492,10 +26424,10 @@
         <v>12</v>
       </c>
       <c r="G92" s="3" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="H92" s="3" t="s">
-        <v>706</v>
+        <v>699</v>
       </c>
     </row>
     <row r="93" spans="1:8" ht="72">
@@ -26521,7 +26453,7 @@
         <v>219</v>
       </c>
       <c r="H93" s="3" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
     </row>
     <row r="94" spans="1:8" ht="72">
@@ -26547,7 +26479,7 @@
         <v>221</v>
       </c>
       <c r="H94" s="3" t="s">
-        <v>707</v>
+        <v>700</v>
       </c>
     </row>
     <row r="95" spans="1:8">
@@ -26599,7 +26531,7 @@
         <v>226</v>
       </c>
       <c r="H96" s="3" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
     </row>
     <row r="97" spans="1:8">
@@ -26625,7 +26557,7 @@
         <v>228</v>
       </c>
       <c r="H97" s="6" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
     </row>
     <row r="98" spans="1:8">
@@ -26651,7 +26583,7 @@
         <v>230</v>
       </c>
       <c r="H98" s="6" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
     </row>
     <row r="99" spans="1:8" ht="201.6">
@@ -26677,7 +26609,7 @@
         <v>233</v>
       </c>
       <c r="H99" s="3" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
     </row>
     <row r="100" spans="1:8" ht="28.8">
@@ -26703,7 +26635,7 @@
         <v>236</v>
       </c>
       <c r="H100" s="6" t="s">
-        <v>708</v>
+        <v>701</v>
       </c>
     </row>
     <row r="101" spans="1:8" ht="129.6">
@@ -26729,7 +26661,7 @@
         <v>238</v>
       </c>
       <c r="H101" s="3" t="s">
-        <v>763</v>
+        <v>754</v>
       </c>
     </row>
     <row r="102" spans="1:8" ht="86.4">
@@ -26755,7 +26687,7 @@
         <v>241</v>
       </c>
       <c r="H102" s="3" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
     </row>
     <row r="103" spans="1:8" ht="302.39999999999998">
@@ -26781,7 +26713,7 @@
         <v>243</v>
       </c>
       <c r="H103" s="3" t="s">
-        <v>728</v>
+        <v>719</v>
       </c>
     </row>
     <row r="104" spans="1:8" ht="28.8">
@@ -26807,7 +26739,7 @@
         <v>246</v>
       </c>
       <c r="H104" s="3" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
     </row>
     <row r="105" spans="1:8" ht="86.4">
@@ -26833,7 +26765,7 @@
         <v>248</v>
       </c>
       <c r="H105" s="3" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
     </row>
     <row r="106" spans="1:8">
@@ -26885,7 +26817,7 @@
         <v>253</v>
       </c>
       <c r="H107" s="6" t="s">
-        <v>630</v>
+        <v>627</v>
       </c>
     </row>
     <row r="108" spans="1:8">
@@ -26937,7 +26869,7 @@
         <v>258</v>
       </c>
       <c r="H109" s="6" t="s">
-        <v>645</v>
+        <v>802</v>
       </c>
     </row>
     <row r="110" spans="1:8">
@@ -27015,7 +26947,7 @@
         <v>266</v>
       </c>
       <c r="H112" s="6" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
     </row>
     <row r="113" spans="1:8" ht="43.2">
@@ -27041,7 +26973,7 @@
         <v>269</v>
       </c>
       <c r="H113" s="3" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
     </row>
     <row r="114" spans="1:8" ht="86.4">
@@ -27064,10 +26996,10 @@
         <v>12</v>
       </c>
       <c r="G114" s="8" t="s">
-        <v>722</v>
+        <v>714</v>
       </c>
       <c r="H114" s="3" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
     </row>
     <row r="115" spans="1:8">
@@ -27093,7 +27025,7 @@
         <v>272</v>
       </c>
       <c r="H115" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
     </row>
     <row r="116" spans="1:8">
@@ -27119,7 +27051,7 @@
         <v>274</v>
       </c>
       <c r="H116" t="s">
-        <v>635</v>
+        <v>632</v>
       </c>
     </row>
     <row r="117" spans="1:8">
@@ -27145,7 +27077,7 @@
         <v>276</v>
       </c>
       <c r="H117" t="s">
-        <v>646</v>
+        <v>803</v>
       </c>
     </row>
     <row r="118" spans="1:8">
@@ -27171,7 +27103,7 @@
         <v>278</v>
       </c>
       <c r="H118" s="6" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
     </row>
     <row r="119" spans="1:8" ht="43.2">
@@ -27197,7 +27129,7 @@
         <v>280</v>
       </c>
       <c r="H119" s="6" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
     </row>
     <row r="120" spans="1:8" ht="28.8">
@@ -27275,7 +27207,7 @@
         <v>288</v>
       </c>
       <c r="H122" s="6" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
     </row>
     <row r="123" spans="1:8" ht="28.8">
@@ -27301,7 +27233,7 @@
         <v>291</v>
       </c>
       <c r="H123" s="3" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
     </row>
     <row r="124" spans="1:8">
@@ -27327,7 +27259,7 @@
         <v>293</v>
       </c>
       <c r="H124" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
     </row>
     <row r="125" spans="1:8" ht="86.4">
@@ -27353,7 +27285,7 @@
         <v>296</v>
       </c>
       <c r="H125" s="3" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
     </row>
     <row r="126" spans="1:8" ht="28.8">
@@ -27379,7 +27311,7 @@
         <v>298</v>
       </c>
       <c r="H126" s="6" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
     </row>
     <row r="127" spans="1:8" ht="28.8">
@@ -27405,7 +27337,7 @@
         <v>300</v>
       </c>
       <c r="H127" s="8" t="s">
-        <v>710</v>
+        <v>703</v>
       </c>
     </row>
     <row r="128" spans="1:8" ht="28.8">
@@ -27431,7 +27363,7 @@
         <v>302</v>
       </c>
       <c r="H128" s="8" t="s">
-        <v>723</v>
+        <v>715</v>
       </c>
     </row>
     <row r="129" spans="1:8" ht="28.8">
@@ -27457,10 +27389,10 @@
         <v>304</v>
       </c>
       <c r="H129" s="8" t="s">
-        <v>711</v>
+        <v>804</v>
       </c>
     </row>
-    <row r="130" spans="1:8">
+    <row r="130" spans="1:8" ht="28.8">
       <c r="A130" s="2" t="s">
         <v>8</v>
       </c>
@@ -27483,7 +27415,7 @@
         <v>306</v>
       </c>
       <c r="H130" s="8" t="s">
-        <v>647</v>
+        <v>805</v>
       </c>
     </row>
     <row r="131" spans="1:8">
@@ -27535,7 +27467,7 @@
         <v>311</v>
       </c>
       <c r="H132" s="3" t="s">
-        <v>709</v>
+        <v>702</v>
       </c>
     </row>
     <row r="133" spans="1:8">
@@ -27561,7 +27493,7 @@
         <v>313</v>
       </c>
       <c r="H133" s="3" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
     </row>
     <row r="134" spans="1:8" ht="28.8">
@@ -27587,7 +27519,7 @@
         <v>316</v>
       </c>
       <c r="H134" s="6" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
     </row>
     <row r="135" spans="1:8" ht="403.2">
@@ -27613,7 +27545,7 @@
         <v>318</v>
       </c>
       <c r="H135" s="3" t="s">
-        <v>736</v>
+        <v>727</v>
       </c>
     </row>
     <row r="136" spans="1:8">
@@ -27639,7 +27571,7 @@
         <v>321</v>
       </c>
       <c r="H136" s="6" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
     </row>
     <row r="137" spans="1:8" ht="43.2">
@@ -27653,7 +27585,7 @@
         <v>1</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>772</v>
+        <v>763</v>
       </c>
       <c r="E137" s="2" t="s">
         <v>11</v>
@@ -27662,10 +27594,10 @@
         <v>12</v>
       </c>
       <c r="G137" s="3" t="s">
-        <v>773</v>
+        <v>764</v>
       </c>
       <c r="H137" s="6" t="s">
-        <v>771</v>
+        <v>762</v>
       </c>
     </row>
     <row r="138" spans="1:8" ht="100.8">
@@ -27679,7 +27611,7 @@
         <v>2</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>733</v>
+        <v>724</v>
       </c>
       <c r="E138" s="2" t="s">
         <v>11</v>
@@ -27688,24 +27620,24 @@
         <v>12</v>
       </c>
       <c r="G138" s="3" t="s">
-        <v>734</v>
+        <v>725</v>
       </c>
       <c r="H138" s="3" t="s">
-        <v>712</v>
+        <v>704</v>
       </c>
     </row>
     <row r="139" spans="1:8" ht="115.2">
       <c r="A139" s="2" t="s">
-        <v>742</v>
+        <v>733</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>752</v>
+        <v>743</v>
       </c>
       <c r="C139" s="2">
         <v>0</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>753</v>
+        <v>744</v>
       </c>
       <c r="E139" s="2" t="s">
         <v>11</v>
@@ -27714,10 +27646,10 @@
         <v>12</v>
       </c>
       <c r="G139" s="3" t="s">
-        <v>754</v>
+        <v>745</v>
       </c>
       <c r="H139" s="3" t="s">
-        <v>755</v>
+        <v>746</v>
       </c>
     </row>
     <row r="140" spans="1:8" ht="409.6">
@@ -27743,7 +27675,7 @@
         <v>323</v>
       </c>
       <c r="H140" s="3" t="s">
-        <v>764</v>
+        <v>755</v>
       </c>
     </row>
     <row r="141" spans="1:8" ht="28.8">
@@ -27769,7 +27701,7 @@
         <v>326</v>
       </c>
       <c r="H141" s="6" t="s">
-        <v>649</v>
+        <v>643</v>
       </c>
     </row>
     <row r="142" spans="1:8">
@@ -27795,7 +27727,7 @@
         <v>329</v>
       </c>
       <c r="H142" s="6" t="s">
-        <v>650</v>
+        <v>644</v>
       </c>
     </row>
     <row r="143" spans="1:8" ht="57.6">
@@ -27821,7 +27753,7 @@
         <v>331</v>
       </c>
       <c r="H143" s="6" t="s">
-        <v>651</v>
+        <v>645</v>
       </c>
     </row>
     <row r="144" spans="1:8">
@@ -27847,7 +27779,7 @@
         <v>333</v>
       </c>
       <c r="H144" s="6" t="s">
-        <v>652</v>
+        <v>646</v>
       </c>
     </row>
     <row r="145" spans="1:8" ht="43.2">
@@ -27873,7 +27805,7 @@
         <v>335</v>
       </c>
       <c r="H145" s="6" t="s">
-        <v>653</v>
+        <v>647</v>
       </c>
     </row>
     <row r="146" spans="1:8" ht="86.4">
@@ -27899,7 +27831,7 @@
         <v>337</v>
       </c>
       <c r="H146" s="3" t="s">
-        <v>654</v>
+        <v>648</v>
       </c>
     </row>
     <row r="147" spans="1:8" ht="216">
@@ -27925,7 +27857,7 @@
         <v>339</v>
       </c>
       <c r="H147" s="3" t="s">
-        <v>655</v>
+        <v>649</v>
       </c>
     </row>
     <row r="148" spans="1:8" ht="86.4">
@@ -27977,7 +27909,7 @@
         <v>345</v>
       </c>
       <c r="H149" s="3" t="s">
-        <v>758</v>
+        <v>749</v>
       </c>
     </row>
     <row r="150" spans="1:8">
@@ -28029,7 +27961,7 @@
         <v>351</v>
       </c>
       <c r="H151" s="3" t="s">
-        <v>656</v>
+        <v>650</v>
       </c>
     </row>
     <row r="152" spans="1:8" ht="28.8">
@@ -28055,7 +27987,7 @@
         <v>354</v>
       </c>
       <c r="H152" s="3" t="s">
-        <v>657</v>
+        <v>651</v>
       </c>
     </row>
     <row r="153" spans="1:8">
@@ -28081,7 +28013,7 @@
         <v>356</v>
       </c>
       <c r="H153" s="3" t="s">
-        <v>658</v>
+        <v>652</v>
       </c>
     </row>
     <row r="154" spans="1:8" ht="129.6">
@@ -28107,7 +28039,7 @@
         <v>359</v>
       </c>
       <c r="H154" s="3" t="s">
-        <v>737</v>
+        <v>728</v>
       </c>
     </row>
     <row r="155" spans="1:8" ht="28.8">
@@ -28185,7 +28117,7 @@
         <v>368</v>
       </c>
       <c r="H157" s="3" t="s">
-        <v>659</v>
+        <v>653</v>
       </c>
     </row>
     <row r="158" spans="1:8" ht="28.8">
@@ -28211,7 +28143,7 @@
         <v>371</v>
       </c>
       <c r="H158" s="6" t="s">
-        <v>660</v>
+        <v>654</v>
       </c>
     </row>
     <row r="159" spans="1:8" ht="409.6">
@@ -28237,7 +28169,7 @@
         <v>373</v>
       </c>
       <c r="H159" s="3" t="s">
-        <v>713</v>
+        <v>705</v>
       </c>
     </row>
     <row r="160" spans="1:8" ht="43.2">
@@ -28263,7 +28195,7 @@
         <v>376</v>
       </c>
       <c r="H160" s="6" t="s">
-        <v>661</v>
+        <v>655</v>
       </c>
     </row>
     <row r="161" spans="1:8" ht="86.4">
@@ -28341,7 +28273,7 @@
         <v>385</v>
       </c>
       <c r="H163" s="6" t="s">
-        <v>714</v>
+        <v>706</v>
       </c>
     </row>
     <row r="164" spans="1:8" ht="100.8">
@@ -28367,7 +28299,7 @@
         <v>388</v>
       </c>
       <c r="H164" s="3" t="s">
-        <v>662</v>
+        <v>656</v>
       </c>
     </row>
     <row r="165" spans="1:8" ht="144">
@@ -28393,7 +28325,7 @@
         <v>390</v>
       </c>
       <c r="H165" s="3" t="s">
-        <v>715</v>
+        <v>707</v>
       </c>
     </row>
     <row r="166" spans="1:8" ht="100.8">
@@ -28419,7 +28351,7 @@
         <v>393</v>
       </c>
       <c r="H166" s="3" t="s">
-        <v>663</v>
+        <v>657</v>
       </c>
     </row>
     <row r="167" spans="1:8" ht="43.2">
@@ -28445,7 +28377,7 @@
         <v>395</v>
       </c>
       <c r="H167" s="6" t="s">
-        <v>664</v>
+        <v>658</v>
       </c>
     </row>
     <row r="168" spans="1:8" ht="115.2">
@@ -28471,7 +28403,7 @@
         <v>398</v>
       </c>
       <c r="H168" s="3" t="s">
-        <v>665</v>
+        <v>659</v>
       </c>
     </row>
     <row r="169" spans="1:8" ht="86.4">
@@ -28549,7 +28481,7 @@
         <v>408</v>
       </c>
       <c r="H171" s="3" t="s">
-        <v>716</v>
+        <v>708</v>
       </c>
     </row>
     <row r="172" spans="1:8" ht="57.6">
@@ -28601,7 +28533,7 @@
         <v>413</v>
       </c>
       <c r="H173" s="3" t="s">
-        <v>675</v>
+        <v>669</v>
       </c>
     </row>
     <row r="174" spans="1:8" ht="57.6">
@@ -28627,7 +28559,7 @@
         <v>416</v>
       </c>
       <c r="H174" s="6" t="s">
-        <v>676</v>
+        <v>670</v>
       </c>
     </row>
     <row r="175" spans="1:8" ht="28.8">
@@ -28702,10 +28634,10 @@
         <v>12</v>
       </c>
       <c r="G177" s="3" t="s">
-        <v>677</v>
+        <v>671</v>
       </c>
       <c r="H177" s="3" t="s">
-        <v>717</v>
+        <v>709</v>
       </c>
     </row>
     <row r="178" spans="1:8" ht="28.8">
@@ -28745,7 +28677,7 @@
         <v>1</v>
       </c>
       <c r="D179" s="2" t="s">
-        <v>768</v>
+        <v>759</v>
       </c>
       <c r="E179" s="2" t="s">
         <v>11</v>
@@ -28754,10 +28686,10 @@
         <v>12</v>
       </c>
       <c r="G179" s="3" t="s">
-        <v>769</v>
+        <v>760</v>
       </c>
       <c r="H179" s="3" t="s">
-        <v>770</v>
+        <v>761</v>
       </c>
     </row>
     <row r="180" spans="1:8" ht="201.6">
@@ -28783,7 +28715,7 @@
         <v>430</v>
       </c>
       <c r="H180" s="3" t="s">
-        <v>746</v>
+        <v>737</v>
       </c>
     </row>
     <row r="181" spans="1:8" ht="86.4">
@@ -28809,7 +28741,7 @@
         <v>433</v>
       </c>
       <c r="H181" s="3" t="s">
-        <v>738</v>
+        <v>729</v>
       </c>
     </row>
     <row r="182" spans="1:8">
@@ -28861,7 +28793,7 @@
         <v>439</v>
       </c>
       <c r="H183" s="6" t="s">
-        <v>681</v>
+        <v>675</v>
       </c>
     </row>
     <row r="184" spans="1:8">
@@ -28887,7 +28819,7 @@
         <v>442</v>
       </c>
       <c r="H184" s="6" t="s">
-        <v>678</v>
+        <v>672</v>
       </c>
     </row>
     <row r="185" spans="1:8">
@@ -28913,7 +28845,7 @@
         <v>445</v>
       </c>
       <c r="H185" s="6" t="s">
-        <v>679</v>
+        <v>673</v>
       </c>
     </row>
     <row r="186" spans="1:8">
@@ -28939,7 +28871,7 @@
         <v>448</v>
       </c>
       <c r="H186" s="6" t="s">
-        <v>682</v>
+        <v>676</v>
       </c>
     </row>
     <row r="187" spans="1:8">
@@ -28965,7 +28897,7 @@
         <v>451</v>
       </c>
       <c r="H187" s="6" t="s">
-        <v>680</v>
+        <v>674</v>
       </c>
     </row>
     <row r="188" spans="1:8" ht="144">
@@ -28991,7 +28923,7 @@
         <v>454</v>
       </c>
       <c r="H188" s="3" t="s">
-        <v>683</v>
+        <v>677</v>
       </c>
     </row>
     <row r="189" spans="1:8" ht="28.8">
@@ -29225,7 +29157,7 @@
         <v>480</v>
       </c>
       <c r="H197" s="6" t="s">
-        <v>684</v>
+        <v>678</v>
       </c>
     </row>
     <row r="198" spans="1:8">
@@ -29303,7 +29235,7 @@
         <v>488</v>
       </c>
       <c r="H200" t="s">
-        <v>718</v>
+        <v>710</v>
       </c>
     </row>
     <row r="201" spans="1:8">
@@ -29329,7 +29261,7 @@
         <v>490</v>
       </c>
       <c r="H201" s="6" t="s">
-        <v>719</v>
+        <v>711</v>
       </c>
     </row>
     <row r="202" spans="1:8" ht="100.8">
@@ -29355,7 +29287,7 @@
         <v>492</v>
       </c>
       <c r="H202" s="3" t="s">
-        <v>739</v>
+        <v>730</v>
       </c>
     </row>
     <row r="203" spans="1:8" ht="158.4">
@@ -29381,7 +29313,7 @@
         <v>494</v>
       </c>
       <c r="H203" s="3" t="s">
-        <v>685</v>
+        <v>679</v>
       </c>
     </row>
     <row r="204" spans="1:8" ht="43.2">
@@ -29407,7 +29339,7 @@
         <v>496</v>
       </c>
       <c r="H204" s="3" t="s">
-        <v>686</v>
+        <v>680</v>
       </c>
     </row>
     <row r="205" spans="1:8" ht="100.8">
@@ -29433,7 +29365,7 @@
         <v>498</v>
       </c>
       <c r="H205" s="3" t="s">
-        <v>687</v>
+        <v>681</v>
       </c>
     </row>
     <row r="206" spans="1:8" ht="43.2">
@@ -29459,7 +29391,7 @@
         <v>500</v>
       </c>
       <c r="H206" s="3" t="s">
-        <v>688</v>
+        <v>682</v>
       </c>
     </row>
     <row r="207" spans="1:8" ht="100.8">
@@ -29485,7 +29417,7 @@
         <v>502</v>
       </c>
       <c r="H207" s="3" t="s">
-        <v>689</v>
+        <v>683</v>
       </c>
     </row>
     <row r="208" spans="1:8" ht="100.8">
@@ -29511,7 +29443,7 @@
         <v>504</v>
       </c>
       <c r="H208" s="3" t="s">
-        <v>720</v>
+        <v>712</v>
       </c>
     </row>
     <row r="209" spans="1:9" ht="115.2">
@@ -29537,7 +29469,7 @@
         <v>506</v>
       </c>
       <c r="H209" s="3" t="s">
-        <v>690</v>
+        <v>684</v>
       </c>
     </row>
     <row r="210" spans="1:9" ht="158.4">
@@ -29563,7 +29495,7 @@
         <v>508</v>
       </c>
       <c r="H210" s="3" t="s">
-        <v>691</v>
+        <v>685</v>
       </c>
     </row>
     <row r="211" spans="1:9" ht="172.8">
@@ -29589,7 +29521,7 @@
         <v>510</v>
       </c>
       <c r="H211" s="3" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="212" spans="1:9" ht="115.2">
@@ -29615,7 +29547,7 @@
         <v>512</v>
       </c>
       <c r="H212" s="3" t="s">
-        <v>693</v>
+        <v>687</v>
       </c>
     </row>
     <row r="213" spans="1:9" ht="158.4">
@@ -29638,10 +29570,10 @@
         <v>12</v>
       </c>
       <c r="G213" s="3" t="s">
-        <v>740</v>
+        <v>731</v>
       </c>
       <c r="H213" s="3" t="s">
-        <v>741</v>
+        <v>732</v>
       </c>
     </row>
     <row r="214" spans="1:9" ht="158.4">
@@ -29667,7 +29599,7 @@
         <v>515</v>
       </c>
       <c r="H214" s="3" t="s">
-        <v>694</v>
+        <v>688</v>
       </c>
     </row>
     <row r="215" spans="1:9" ht="187.2">
@@ -29681,7 +29613,7 @@
         <v>16</v>
       </c>
       <c r="D215" s="2" t="s">
-        <v>801</v>
+        <v>790</v>
       </c>
       <c r="E215" s="2" t="s">
         <v>11</v>
@@ -29690,10 +29622,10 @@
         <v>12</v>
       </c>
       <c r="G215" s="3" t="s">
-        <v>803</v>
+        <v>792</v>
       </c>
       <c r="H215" s="3" t="s">
-        <v>804</v>
+        <v>793</v>
       </c>
     </row>
     <row r="216" spans="1:9" ht="187.2">
@@ -29707,7 +29639,7 @@
         <v>17</v>
       </c>
       <c r="D216" s="2" t="s">
-        <v>802</v>
+        <v>791</v>
       </c>
       <c r="E216" s="2" t="s">
         <v>11</v>
@@ -29716,10 +29648,10 @@
         <v>12</v>
       </c>
       <c r="G216" s="3" t="s">
-        <v>805</v>
+        <v>794</v>
       </c>
       <c r="H216" s="3" t="s">
-        <v>806</v>
+        <v>795</v>
       </c>
     </row>
     <row r="217" spans="1:9" ht="100.8">
@@ -29733,7 +29665,7 @@
         <v>18</v>
       </c>
       <c r="D217" s="2" t="s">
-        <v>795</v>
+        <v>784</v>
       </c>
       <c r="E217" s="2" t="s">
         <v>11</v>
@@ -29742,10 +29674,10 @@
         <v>12</v>
       </c>
       <c r="G217" s="3" t="s">
-        <v>796</v>
+        <v>785</v>
       </c>
       <c r="H217" s="3" t="s">
-        <v>799</v>
+        <v>788</v>
       </c>
     </row>
     <row r="218" spans="1:9" ht="100.8">
@@ -29759,7 +29691,7 @@
         <v>19</v>
       </c>
       <c r="D218" s="2" t="s">
-        <v>797</v>
+        <v>786</v>
       </c>
       <c r="E218" s="2" t="s">
         <v>11</v>
@@ -29768,10 +29700,10 @@
         <v>12</v>
       </c>
       <c r="G218" s="3" t="s">
-        <v>798</v>
+        <v>787</v>
       </c>
       <c r="H218" s="3" t="s">
-        <v>800</v>
+        <v>789</v>
       </c>
     </row>
     <row r="219" spans="1:9" ht="43.2">
@@ -29797,7 +29729,7 @@
         <v>517</v>
       </c>
       <c r="H219" s="3" t="s">
-        <v>695</v>
+        <v>689</v>
       </c>
     </row>
     <row r="220" spans="1:9" ht="409.6">
@@ -29811,7 +29743,7 @@
         <v>21</v>
       </c>
       <c r="D220" s="2" t="s">
-        <v>765</v>
+        <v>756</v>
       </c>
       <c r="E220" s="2" t="s">
         <v>11</v>
@@ -29820,10 +29752,10 @@
         <v>12</v>
       </c>
       <c r="G220" s="3" t="s">
-        <v>766</v>
+        <v>757</v>
       </c>
       <c r="H220" s="3" t="s">
-        <v>767</v>
+        <v>758</v>
       </c>
       <c r="I220" s="3"/>
     </row>
@@ -29850,7 +29782,7 @@
         <v>519</v>
       </c>
       <c r="H221" s="3" t="s">
-        <v>696</v>
+        <v>690</v>
       </c>
     </row>
     <row r="222" spans="1:9" ht="43.2">
@@ -29902,7 +29834,7 @@
         <v>524</v>
       </c>
       <c r="H223" s="3" t="s">
-        <v>666</v>
+        <v>660</v>
       </c>
     </row>
     <row r="224" spans="1:9" ht="115.2">
@@ -29928,7 +29860,7 @@
         <v>526</v>
       </c>
       <c r="H224" s="3" t="s">
-        <v>667</v>
+        <v>661</v>
       </c>
     </row>
     <row r="225" spans="1:8" ht="43.2">
@@ -29954,7 +29886,7 @@
         <v>528</v>
       </c>
       <c r="H225" s="3" t="s">
-        <v>668</v>
+        <v>662</v>
       </c>
     </row>
     <row r="226" spans="1:8" ht="100.8">
@@ -29980,7 +29912,7 @@
         <v>530</v>
       </c>
       <c r="H226" s="3" t="s">
-        <v>721</v>
+        <v>713</v>
       </c>
     </row>
     <row r="227" spans="1:8" ht="43.2">
@@ -30032,7 +29964,7 @@
         <v>535</v>
       </c>
       <c r="H228" s="3" t="s">
-        <v>669</v>
+        <v>663</v>
       </c>
     </row>
     <row r="229" spans="1:8" ht="100.8">
@@ -30058,7 +29990,7 @@
         <v>537</v>
       </c>
       <c r="H229" s="3" t="s">
-        <v>670</v>
+        <v>664</v>
       </c>
     </row>
     <row r="230" spans="1:8" ht="28.8">
@@ -30084,7 +30016,7 @@
         <v>540</v>
       </c>
       <c r="H230" s="6" t="s">
-        <v>671</v>
+        <v>665</v>
       </c>
     </row>
     <row r="231" spans="1:8" ht="28.8">
@@ -30136,7 +30068,7 @@
         <v>546</v>
       </c>
       <c r="H232" s="3" t="s">
-        <v>672</v>
+        <v>666</v>
       </c>
     </row>
     <row r="233" spans="1:8" ht="100.8">
@@ -30162,7 +30094,7 @@
         <v>548</v>
       </c>
       <c r="H233" s="3" t="s">
-        <v>673</v>
+        <v>667</v>
       </c>
     </row>
     <row r="234" spans="1:8" ht="43.2">
@@ -30188,7 +30120,7 @@
         <v>550</v>
       </c>
       <c r="H234" s="3" t="s">
-        <v>674</v>
+        <v>668</v>
       </c>
     </row>
     <row r="235" spans="1:8">
@@ -30240,7 +30172,7 @@
         <v>557</v>
       </c>
       <c r="H236" s="6" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="237" spans="1:8" ht="28.8">
@@ -30266,7 +30198,7 @@
         <v>559</v>
       </c>
       <c r="H237" s="6" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
     </row>
     <row r="238" spans="1:8">
@@ -30401,7 +30333,7 @@
     </row>
     <row r="243" spans="1:8">
       <c r="A243" t="s">
-        <v>742</v>
+        <v>733</v>
       </c>
       <c r="B243" t="s">
         <v>572</v>
@@ -30410,7 +30342,7 @@
         <v>1</v>
       </c>
       <c r="D243" t="s">
-        <v>743</v>
+        <v>734</v>
       </c>
       <c r="E243" t="s">
         <v>11</v>
@@ -30419,10 +30351,10 @@
         <v>12</v>
       </c>
       <c r="G243" t="s">
-        <v>744</v>
+        <v>735</v>
       </c>
       <c r="H243" s="4" t="s">
-        <v>745</v>
+        <v>736</v>
       </c>
     </row>
     <row r="244" spans="1:8">

</xml_diff>

<commit_message>
Easy Form product name alignment
</commit_message>
<xml_diff>
--- a/docassemble/PowerOfAttorneyHealthCare/data/sources/poa_hc_es.xlsx
+++ b/docassemble/PowerOfAttorneyHealthCare/data/sources/poa_hc_es.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60905B48-AB5B-4C17-86EE-127EA6AE26FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4C5AF97-BFD9-495E-8DD6-07F1DA8BC7A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-37500" yWindow="-5220" windowWidth="25410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -9895,112 +9895,6 @@
     </r>
   </si>
   <si>
-    <t>53f4eea875cd986be67631969353d829</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if for_yourself == True:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">**Do you want to delay future revocation of this Power of Attorney by 30 days?**
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% else:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">**Does </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${principal.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> want to delay future revocation of this Power of Attorney by 30 days?**
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${word(yesno(delayed_revocation))}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-  </si>
-  <si>
     <t>616bf23d4742bfd429f8eb331950c2c4</t>
   </si>
   <si>
@@ -15675,98 +15569,6 @@
   <si>
     <r>
       <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if for_yourself == True:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">**¿Quieres posponer por 30 días una futura revocación de este Poder Notarial?**
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% else:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">**¿Quiere </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${principal.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> posponer por 30 días una futura revocación de este Poder Notarial?**
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${word(yesno(delayed_revocation))}</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
@@ -16647,86 +16449,6 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> no autorizo una autopsia. (on behalf of principal) no autoriza una autopsia.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if for_yourself == True:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">¿Quieres posponer una futura revocación de este poder notarial por 30 días?
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% else:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">¿Quiere </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${principal.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> posponer una futura revocación de este poder notarial por 30 días?
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>% endif</t>
     </r>
   </si>
   <si>
@@ -18114,90 +17836,6 @@
 </t>
   </si>
   <si>
-    <t>17e34474c2aecb37706af0eba9c1da9e</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if for_yourself == True:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Do you want to delay future revocation of this Power of Attorney by 30 days?
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% else:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Does </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${principal.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> want to delay future revocation of this Power of Attorney by 30 days?
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -18260,248 +17898,6 @@
   <si>
     <r>
       <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if for_yourself == True:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Puedes cambiar de opinión y poner fin a tu Poder Notarial para el Cuidado de la Salud en cualquier momento. Esto se llama revocación.
-La revocación significa que dejas de permitir que </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${agent.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> tome decisiones por ti. Para obtener más información, lee el artículo de ILAO sobre [**poner fin a un Poder Notarial**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://es.illinoislegalaid.org/legal-information/ending-power-attorney-0</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>).
-Puedes poner fin a un Poder Notarial haciendo una revocación formal. Para hacer una Revocación de Poder Notarial, usa el [**Formulario Guiado de Revocación de Poder Notarial**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://es.illinoislegalaid.org/legal-information/power-attorney-revocation</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">).
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% else:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${principal.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> puede cambiar de opinión y poner fin a su Poder Notarial para el Cuidado de la Salud en cualquier momento. Esto se llama revocación.
-La revocación significa que </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${principal.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> deja de permitir que </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${agent.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> tome decisiones en su nombre. Para obtener más información, lee el artículo de ILAO sobre [**poner fin a un Poder Notarial**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://es.illinoislegalaid.org/legal-information/ending-power-attorney-0</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">). 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${principal.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> puede poner fin a un Poder Notarial haciendo una revocación formal. Para hacer una Revocación de Poder Notarial, usa el [**Formulario Guiado de Revocación de Poder Notarial**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://es.illinoislegalaid.org/legal-information/power-attorney-revocation</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">).
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>% endif</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
@@ -18543,41 +17939,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Tus formularios están adjuntos.
-¡Gracias por usar los Formularios Guiados de ILAO!
-[Illinois Legal Aid Online](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://es.illinoislegalaid.org</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
       <t xml:space="preserve">**Estás haciendo estos formularios para:**
 </t>
     </r>
@@ -18828,118 +18189,6 @@
   </si>
   <si>
     <t>Acerca del testigo</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if not user_logged_in():
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[${fa_icon("sign-in-alt", color="#0079d0", size="sm")} **Iniciar sesión**]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${url_of('login', next=interview_url())}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>) o [**crear**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${url_of('register', next=interview_url())}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">) una cuenta de Formularios Guiados de ILAO para guardar tu progreso (opcional).
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ action_button_html(interview_url(i="docassemble.ILAO:feedback.yml", easy_form_interview=ilao_easy_form_url, easy_form_title=ilao_easy_form_title, easy_form_page=current_context().question_id, easy_form_variable=current_context().variable, local=False,reset=1), label=':comment: ¿Fue útil este programa?', color="#181c36", size="md", new_window=True) }</t>
-    </r>
   </si>
   <si>
     <r>
@@ -21408,112 +20657,6 @@
 **Note:** The Power of Attorney needs to be signed in front of at least one witness to become official.
 Thank you for using ILAO Easy Forms!
 </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Tus formularios están listos. Puedes verlos y descargarlos abajo. Haz clic en **Hacer cambios** para corregir cualquier error.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">[YOUTUBE vuN6YBYEh6k]
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Lee las instrucciones para saber qué hacer después.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ action_button_html(url_action('review_answers'), label=':edit: Hacer cambios', color='success', size="md") }
-**Nota:** Estos son formularios e instrucciones bilingües en inglés y español. Para obtener formularios solo en inglés, seleccione **English** en el selector de idioma :globe: del menú.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ al_user_bundle.download_list_html() }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-&amp;nbsp;
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ al_user_bundle.send_button_html(show_editable_checkbox=False) }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-**Nota:** El Poder Notarial debe firmarse frente a al menos un testigo para que sea válido.
-¡Gracias por usar los Formularios Guiados de ILAO!</t>
     </r>
   </si>
   <si>
@@ -22962,70 +22105,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">% if get_language() == 'en':
-:globe: English | [Español](${ interview_url(new_session=1, lang="es") })
-% else:
-:globe: [English](${ interview_url(new_session=1, lang="en") }) | Español
-% endif
-Bienvenido(a) al Formulario Guiado de Poder Notarial para el Cuidado de la Salud de Illinois Legal Aid Online.
-Este programa te ayuda a crear documentos que le otorgan a una persona de tu confianza la autoridad legal para tomar decisiones sobre tu atención médica. Esto significa que esa persona podrá tomar decisiones sobre tu atención médica cuando no puedas hacerlo por ti mismo(a). Si así lo deseas, también puedes autorizarla para que tome decisiones sobre tu atención médica antes de que eso ocurra.
-Este programa incluye videos con información sobre cómo hacer un Poder Notarial para el Cuidado de la Salud. No tienes que verlos, pero pueden serte útiles.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">[YOUTUBE ccToVpEse7s]
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Para obtener más información, lee el artículo de ILAO sobre los [**Conceptos Básicos del Poder Notarial para el Cuidado de la Salud**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://es.illinoislegalaid.org/legal-information/setting-power-attorney-healthcare</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>).</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
       <t xml:space="preserve">Este programa no ofrece asesoramiento legal. No sustituye al asesoramiento de un abogado.
 El uso de este programa no crea una relación abogado-cliente entre ti e Illinois Legal Aid Online ni sus empleados.
 Los videos en este programa ofrecen información importante sobre el proceso de planificación anticipada. Proporcionan únicamente información, no asesoramiento legal. No crean una relación abogado-cliente entre ti y el Center for Disability and Elder Law ni sus empleados.
@@ -23560,6 +22639,885 @@
   </si>
   <si>
     <t>Ingresa la dirección de ${agent.name_full()} a continuación.</t>
+  </si>
+  <si>
+    <t>7adb8cda094fcb1e943e8289b835d423</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if for_yourself == True:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Do you want a future revocation of this Power of Attorney to take effect 30 days after you revoke it?
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% else:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Does </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> want a future revocation of this Power of Attorney to take effect 30 days after they revoke it?
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if for_yourself == True:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">¿Quieres retrasar por 30 días los efectos de una futura revocación de este poder notarial?
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% else:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">¿Quiere ${principal.name_full()} retrasar por 30 días los efectos de una futura revocación de este poder notarial?
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>% endif</t>
+    </r>
+  </si>
+  <si>
+    <t>b3343595b114509354681fa2fd342721</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if for_yourself == True:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">**Do you want a future revocation of this Power of Attorney to take effect 30 days after you revoke it?**
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% else:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">**Does </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> want a future revocation of this Power of Attorney to take effect 30 days after they revoke it?**      
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${word(yesno(delayed_revocation))}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if for_yourself == True:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">**¿Quieres retrasar por 30 días los efectos de una futura revocación de este poder notarial?**
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% else:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">**¿Quiere ${principal.name_full()} retrasar por 30 días los efectos de una futura revocación de este poder notarial?**
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${word(yesno(delayed_revocation))}</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if get_language() == 'en':
+:globe: English | [Español](${ interview_url(new_session=1, lang="es") })
+% else:
+:globe: [English](${ interview_url(new_session=1, lang="en") }) | Español
+% endif
+Bienvenido(a) al Formulario Fácil de Poder Notarial para el Cuidado de la Salud de Illinois Legal Aid Online.
+Este programa te ayuda a crear documentos que le otorgan a una persona de tu confianza la autoridad legal para tomar decisiones sobre tu atención médica. Esto significa que esa persona podrá tomar decisiones sobre tu atención médica cuando no puedas hacerlo por ti mismo(a). Si así lo deseas, también puedes autorizarla para que tome decisiones sobre tu atención médica antes de que eso ocurra.
+Este programa incluye videos con información sobre cómo hacer un Poder Notarial para el Cuidado de la Salud. No tienes que verlos, pero pueden serte útiles.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">[YOUTUBE ccToVpEse7s]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Para obtener más información, lee el artículo de ILAO sobre los [**Conceptos Básicos del Poder Notarial para el Cuidado de la Salud**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://es.illinoislegalaid.org/legal-information/setting-power-attorney-healthcare</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if for_yourself == True:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Puedes cambiar de opinión y poner fin a tu Poder Notarial para el Cuidado de la Salud en cualquier momento. Esto se llama revocación.
+La revocación significa que dejas de permitir que </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${agent.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> tome decisiones por ti. Para obtener más información, lee el artículo de ILAO sobre [**poner fin a un Poder Notarial**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://es.illinoislegalaid.org/legal-information/ending-power-attorney-0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>).
+Puedes poner fin a un Poder Notarial haciendo una revocación formal. Para hacer una Revocación de Poder Notarial, usa el [**Formulario Fácil de Revocación de Poder Notarial**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://es.illinoislegalaid.org/legal-information/power-attorney-revocation</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% else:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> puede cambiar de opinión y poner fin a su Poder Notarial para el Cuidado de la Salud en cualquier momento. Esto se llama revocación.
+La revocación significa que </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> deja de permitir que </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${agent.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> tome decisiones en su nombre. Para obtener más información, lee el artículo de ILAO sobre [**poner fin a un Poder Notarial**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://es.illinoislegalaid.org/legal-information/ending-power-attorney-0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">). 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> puede poner fin a un Poder Notarial haciendo una revocación formal. Para hacer una Revocación de Poder Notarial, usa el [**Formulario Fácil de Revocación de Poder Notarial**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://es.illinoislegalaid.org/legal-information/power-attorney-revocation</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>% endif</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Tus formularios están listos. Puedes verlos y descargarlos abajo. Haz clic en **Hacer cambios** para corregir cualquier error.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">[YOUTUBE vuN6YBYEh6k]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Lee las instrucciones para saber qué hacer después.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ action_button_html(url_action('review_answers'), label=':edit: Hacer cambios', color='success', size="md") }
+**Nota:** Estos son formularios e instrucciones bilingües en inglés y español. Para obtener formularios solo en inglés, seleccione **English** en el selector de idioma :globe: del menú.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ al_user_bundle.download_list_html() }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+&amp;nbsp;
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ al_user_bundle.send_button_html(show_editable_checkbox=False) }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+**Nota:** El Poder Notarial debe firmarse frente a al menos un testigo para que sea válido.
+¡Gracias por usar los Formularios Fáciles de ILAO!</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if not user_logged_in():
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[${fa_icon("sign-in-alt", color="#0079d0", size="sm")} **Iniciar sesión**]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${url_of('login', next=interview_url())}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) o [**crear**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${url_of('register', next=interview_url())}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">) una cuenta de Formularios Fáciles de ILAO para guardar tu progreso (opcional).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ action_button_html(interview_url(i="docassemble.ILAO:feedback.yml", easy_form_interview=ilao_easy_form_url, easy_form_title=ilao_easy_form_title, easy_form_page=current_context().question_id, easy_form_variable=current_context().variable, local=False,reset=1), label=':comment: ¿Fue útil este programa?', color="#181c36", size="md", new_window=True) }</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Tus formularios están adjuntos.
+¡Gracias por usar los Formularios Fáciles de ILAO!
+[Illinois Legal Aid Online](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://es.illinoislegalaid.org</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -24101,7 +24059,7 @@
         <v>1</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>765</v>
+        <v>755</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>11</v>
@@ -24110,10 +24068,10 @@
         <v>12</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>766</v>
+        <v>756</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>796</v>
+        <v>802</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -24165,7 +24123,7 @@
         <v>20</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -24269,7 +24227,7 @@
         <v>31</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>798</v>
+        <v>787</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="28.8">
@@ -24283,7 +24241,7 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>720</v>
+        <v>716</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>11</v>
@@ -24292,7 +24250,7 @@
         <v>12</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>723</v>
+        <v>719</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>33</v>
@@ -24309,7 +24267,7 @@
         <v>1</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>721</v>
+        <v>717</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>11</v>
@@ -24318,7 +24276,7 @@
         <v>12</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>722</v>
+        <v>718</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>34</v>
@@ -24335,7 +24293,7 @@
         <v>0</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>773</v>
+        <v>763</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>11</v>
@@ -24344,10 +24302,10 @@
         <v>12</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>774</v>
+        <v>764</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>777</v>
+        <v>767</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="216">
@@ -24361,7 +24319,7 @@
         <v>1</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>775</v>
+        <v>765</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>11</v>
@@ -24370,10 +24328,10 @@
         <v>12</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>776</v>
+        <v>766</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>778</v>
+        <v>768</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="28.8">
@@ -24425,7 +24383,7 @@
         <v>41</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>738</v>
+        <v>729</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="28.8">
@@ -24477,21 +24435,21 @@
         <v>47</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>726</v>
+        <v>720</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="115.2">
       <c r="A18" s="2" t="s">
-        <v>733</v>
+        <v>725</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>739</v>
+        <v>730</v>
       </c>
       <c r="C18" s="2">
         <v>0</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>740</v>
+        <v>731</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>11</v>
@@ -24500,18 +24458,18 @@
         <v>12</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>741</v>
+        <v>732</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>742</v>
+        <v>733</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="28.8">
       <c r="A19" s="2" t="s">
-        <v>733</v>
+        <v>725</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>739</v>
+        <v>730</v>
       </c>
       <c r="C19" s="2">
         <v>1</v>
@@ -24555,7 +24513,7 @@
         <v>53</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>797</v>
+        <v>786</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -24581,7 +24539,7 @@
         <v>56</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="43.2">
@@ -24607,7 +24565,7 @@
         <v>58</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>716</v>
+        <v>712</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="57.6">
@@ -24633,7 +24591,7 @@
         <v>60</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>717</v>
+        <v>713</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="28.8">
@@ -24659,7 +24617,7 @@
         <v>62</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="57.6">
@@ -24685,12 +24643,12 @@
         <v>64</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26" s="2" t="s">
-        <v>733</v>
+        <v>725</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>54</v>
@@ -24699,7 +24657,7 @@
         <v>5</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>767</v>
+        <v>757</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>11</v>
@@ -24708,15 +24666,15 @@
         <v>12</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>768</v>
+        <v>758</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>771</v>
+        <v>761</v>
       </c>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="2" t="s">
-        <v>733</v>
+        <v>725</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>54</v>
@@ -24725,7 +24683,7 @@
         <v>6</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>769</v>
+        <v>759</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>11</v>
@@ -24734,10 +24692,10 @@
         <v>12</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>770</v>
+        <v>760</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>772</v>
+        <v>762</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="28.8">
@@ -24763,7 +24721,7 @@
         <v>67</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="244.8">
@@ -24789,7 +24747,7 @@
         <v>69</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="86.4">
@@ -24815,7 +24773,7 @@
         <v>72</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="409.6">
@@ -24829,7 +24787,7 @@
         <v>1</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>750</v>
+        <v>741</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>11</v>
@@ -24838,10 +24796,10 @@
         <v>12</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>751</v>
+        <v>742</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>752</v>
+        <v>743</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -24867,7 +24825,7 @@
         <v>74</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -24893,7 +24851,7 @@
         <v>76</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -24919,7 +24877,7 @@
         <v>78</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -24945,7 +24903,7 @@
         <v>80</v>
       </c>
       <c r="H35" s="8" t="s">
-        <v>747</v>
+        <v>738</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -24997,7 +24955,7 @@
         <v>85</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="100.8">
@@ -25023,7 +24981,7 @@
         <v>88</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="28.8">
@@ -25049,7 +25007,7 @@
         <v>90</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="86.4">
@@ -25075,7 +25033,7 @@
         <v>93</v>
       </c>
       <c r="H40" s="10" t="s">
-        <v>799</v>
+        <v>788</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="28.8">
@@ -25101,7 +25059,7 @@
         <v>96</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="144">
@@ -25127,7 +25085,7 @@
         <v>98</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="86.4">
@@ -25179,7 +25137,7 @@
         <v>105</v>
       </c>
       <c r="H44" s="3" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="374.4">
@@ -25205,7 +25163,7 @@
         <v>107</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>800</v>
+        <v>789</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="86.4">
@@ -25231,7 +25189,7 @@
         <v>110</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="28.8">
@@ -25257,7 +25215,7 @@
         <v>112</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="28.8">
@@ -25283,7 +25241,7 @@
         <v>115</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>691</v>
+        <v>688</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -25309,7 +25267,7 @@
         <v>117</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="43.2">
@@ -25335,12 +25293,12 @@
         <v>119</v>
       </c>
       <c r="H50" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="28.8">
       <c r="A51" s="2" t="s">
-        <v>733</v>
+        <v>725</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>113</v>
@@ -25349,7 +25307,7 @@
         <v>4</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>782</v>
+        <v>772</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>11</v>
@@ -25358,10 +25316,10 @@
         <v>12</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>783</v>
+        <v>773</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>806</v>
+        <v>795</v>
       </c>
     </row>
     <row r="52" spans="1:8">
@@ -25387,7 +25345,7 @@
         <v>121</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
     </row>
     <row r="53" spans="1:8">
@@ -25413,7 +25371,7 @@
         <v>123</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
     </row>
     <row r="54" spans="1:8" ht="129.6">
@@ -25427,7 +25385,7 @@
         <v>0</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>779</v>
+        <v>769</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>11</v>
@@ -25436,10 +25394,10 @@
         <v>12</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>780</v>
+        <v>770</v>
       </c>
       <c r="H54" s="3" t="s">
-        <v>781</v>
+        <v>771</v>
       </c>
     </row>
     <row r="55" spans="1:8" ht="28.8">
@@ -25465,7 +25423,7 @@
         <v>126</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>718</v>
+        <v>714</v>
       </c>
     </row>
     <row r="56" spans="1:8" ht="28.8">
@@ -25517,7 +25475,7 @@
         <v>132</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
     </row>
     <row r="58" spans="1:8" ht="100.8">
@@ -25543,7 +25501,7 @@
         <v>135</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>753</v>
+        <v>744</v>
       </c>
     </row>
     <row r="59" spans="1:8" ht="288">
@@ -25569,7 +25527,7 @@
         <v>137</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>801</v>
+        <v>790</v>
       </c>
     </row>
     <row r="60" spans="1:8" ht="28.8">
@@ -25595,7 +25553,7 @@
         <v>140</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
     </row>
     <row r="61" spans="1:8">
@@ -25647,7 +25605,7 @@
         <v>146</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
     </row>
     <row r="63" spans="1:8" ht="28.8">
@@ -25673,7 +25631,7 @@
         <v>148</v>
       </c>
       <c r="H63" s="3" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
     </row>
     <row r="64" spans="1:8" ht="144">
@@ -25699,7 +25657,7 @@
         <v>150</v>
       </c>
       <c r="H64" s="3" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
     </row>
     <row r="65" spans="1:8">
@@ -25777,7 +25735,7 @@
         <v>158</v>
       </c>
       <c r="H67" s="6" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
     </row>
     <row r="68" spans="1:8" ht="43.2">
@@ -25803,7 +25761,7 @@
         <v>160</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
     </row>
     <row r="69" spans="1:8" ht="57.6">
@@ -25829,7 +25787,7 @@
         <v>162</v>
       </c>
       <c r="H69" s="6" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
     </row>
     <row r="70" spans="1:8">
@@ -25881,7 +25839,7 @@
         <v>168</v>
       </c>
       <c r="H71" s="3" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
     </row>
     <row r="72" spans="1:8" ht="172.8">
@@ -25907,7 +25865,7 @@
         <v>170</v>
       </c>
       <c r="H72" s="3" t="s">
-        <v>692</v>
+        <v>689</v>
       </c>
     </row>
     <row r="73" spans="1:8" ht="28.8">
@@ -25933,7 +25891,7 @@
         <v>172</v>
       </c>
       <c r="H73" s="9" t="s">
-        <v>693</v>
+        <v>690</v>
       </c>
     </row>
     <row r="74" spans="1:8">
@@ -25959,7 +25917,7 @@
         <v>174</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="43.2">
@@ -25985,7 +25943,7 @@
         <v>176</v>
       </c>
       <c r="H75" s="3" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
     </row>
     <row r="76" spans="1:8" ht="57.6">
@@ -26011,7 +25969,7 @@
         <v>178</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>695</v>
+        <v>692</v>
       </c>
     </row>
     <row r="77" spans="1:8">
@@ -26037,7 +25995,7 @@
         <v>180</v>
       </c>
       <c r="H77" s="3" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
     </row>
     <row r="78" spans="1:8" ht="28.8">
@@ -26089,7 +26047,7 @@
         <v>186</v>
       </c>
       <c r="H79" s="3" t="s">
-        <v>694</v>
+        <v>691</v>
       </c>
     </row>
     <row r="80" spans="1:8" ht="115.2">
@@ -26115,7 +26073,7 @@
         <v>189</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
     </row>
     <row r="81" spans="1:8" ht="360">
@@ -26141,7 +26099,7 @@
         <v>191</v>
       </c>
       <c r="H81" s="3" t="s">
-        <v>696</v>
+        <v>693</v>
       </c>
     </row>
     <row r="82" spans="1:8" ht="28.8">
@@ -26167,7 +26125,7 @@
         <v>194</v>
       </c>
       <c r="H82" s="6" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
     </row>
     <row r="83" spans="1:8" ht="28.8">
@@ -26190,10 +26148,10 @@
         <v>12</v>
       </c>
       <c r="G83" s="3" t="s">
-        <v>748</v>
+        <v>739</v>
       </c>
       <c r="H83" s="3" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
     </row>
     <row r="84" spans="1:8" ht="72">
@@ -26219,7 +26177,7 @@
         <v>198</v>
       </c>
       <c r="H84" s="3" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
     </row>
     <row r="85" spans="1:8" ht="72">
@@ -26245,7 +26203,7 @@
         <v>200</v>
       </c>
       <c r="H85" s="3" t="s">
-        <v>697</v>
+        <v>694</v>
       </c>
     </row>
     <row r="86" spans="1:8">
@@ -26297,7 +26255,7 @@
         <v>205</v>
       </c>
       <c r="H87" s="3" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
     </row>
     <row r="88" spans="1:8">
@@ -26323,7 +26281,7 @@
         <v>207</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
     </row>
     <row r="89" spans="1:8">
@@ -26375,7 +26333,7 @@
         <v>213</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>698</v>
+        <v>695</v>
       </c>
     </row>
     <row r="91" spans="1:8" ht="43.2">
@@ -26401,7 +26359,7 @@
         <v>215</v>
       </c>
       <c r="H91" s="6" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
     </row>
     <row r="92" spans="1:8" ht="43.2">
@@ -26424,10 +26382,10 @@
         <v>12</v>
       </c>
       <c r="G92" s="3" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="H92" s="3" t="s">
-        <v>699</v>
+        <v>696</v>
       </c>
     </row>
     <row r="93" spans="1:8" ht="72">
@@ -26453,7 +26411,7 @@
         <v>219</v>
       </c>
       <c r="H93" s="3" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
     </row>
     <row r="94" spans="1:8" ht="72">
@@ -26479,7 +26437,7 @@
         <v>221</v>
       </c>
       <c r="H94" s="3" t="s">
-        <v>700</v>
+        <v>697</v>
       </c>
     </row>
     <row r="95" spans="1:8">
@@ -26531,7 +26489,7 @@
         <v>226</v>
       </c>
       <c r="H96" s="3" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
     </row>
     <row r="97" spans="1:8">
@@ -26557,7 +26515,7 @@
         <v>228</v>
       </c>
       <c r="H97" s="6" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
     </row>
     <row r="98" spans="1:8">
@@ -26583,7 +26541,7 @@
         <v>230</v>
       </c>
       <c r="H98" s="6" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
     </row>
     <row r="99" spans="1:8" ht="201.6">
@@ -26609,7 +26567,7 @@
         <v>233</v>
       </c>
       <c r="H99" s="3" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
     </row>
     <row r="100" spans="1:8" ht="28.8">
@@ -26635,7 +26593,7 @@
         <v>236</v>
       </c>
       <c r="H100" s="6" t="s">
-        <v>701</v>
+        <v>698</v>
       </c>
     </row>
     <row r="101" spans="1:8" ht="129.6">
@@ -26661,7 +26619,7 @@
         <v>238</v>
       </c>
       <c r="H101" s="3" t="s">
-        <v>754</v>
+        <v>745</v>
       </c>
     </row>
     <row r="102" spans="1:8" ht="86.4">
@@ -26687,7 +26645,7 @@
         <v>241</v>
       </c>
       <c r="H102" s="3" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
     </row>
     <row r="103" spans="1:8" ht="302.39999999999998">
@@ -26713,7 +26671,7 @@
         <v>243</v>
       </c>
       <c r="H103" s="3" t="s">
-        <v>719</v>
+        <v>715</v>
       </c>
     </row>
     <row r="104" spans="1:8" ht="28.8">
@@ -26739,7 +26697,7 @@
         <v>246</v>
       </c>
       <c r="H104" s="3" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
     </row>
     <row r="105" spans="1:8" ht="86.4">
@@ -26765,7 +26723,7 @@
         <v>248</v>
       </c>
       <c r="H105" s="3" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
     </row>
     <row r="106" spans="1:8">
@@ -26817,7 +26775,7 @@
         <v>253</v>
       </c>
       <c r="H107" s="6" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
     </row>
     <row r="108" spans="1:8">
@@ -26869,7 +26827,7 @@
         <v>258</v>
       </c>
       <c r="H109" s="6" t="s">
-        <v>802</v>
+        <v>791</v>
       </c>
     </row>
     <row r="110" spans="1:8">
@@ -26947,7 +26905,7 @@
         <v>266</v>
       </c>
       <c r="H112" s="6" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
     </row>
     <row r="113" spans="1:8" ht="43.2">
@@ -26973,7 +26931,7 @@
         <v>269</v>
       </c>
       <c r="H113" s="3" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
     </row>
     <row r="114" spans="1:8" ht="86.4">
@@ -26996,10 +26954,10 @@
         <v>12</v>
       </c>
       <c r="G114" s="8" t="s">
-        <v>714</v>
+        <v>710</v>
       </c>
       <c r="H114" s="3" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
     </row>
     <row r="115" spans="1:8">
@@ -27025,7 +26983,7 @@
         <v>272</v>
       </c>
       <c r="H115" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
     </row>
     <row r="116" spans="1:8">
@@ -27051,7 +27009,7 @@
         <v>274</v>
       </c>
       <c r="H116" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
     </row>
     <row r="117" spans="1:8">
@@ -27077,7 +27035,7 @@
         <v>276</v>
       </c>
       <c r="H117" t="s">
-        <v>803</v>
+        <v>792</v>
       </c>
     </row>
     <row r="118" spans="1:8">
@@ -27103,7 +27061,7 @@
         <v>278</v>
       </c>
       <c r="H118" s="6" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
     </row>
     <row r="119" spans="1:8" ht="43.2">
@@ -27129,7 +27087,7 @@
         <v>280</v>
       </c>
       <c r="H119" s="6" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
     </row>
     <row r="120" spans="1:8" ht="28.8">
@@ -27207,7 +27165,7 @@
         <v>288</v>
       </c>
       <c r="H122" s="6" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
     </row>
     <row r="123" spans="1:8" ht="28.8">
@@ -27233,7 +27191,7 @@
         <v>291</v>
       </c>
       <c r="H123" s="3" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
     </row>
     <row r="124" spans="1:8">
@@ -27259,7 +27217,7 @@
         <v>293</v>
       </c>
       <c r="H124" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
     </row>
     <row r="125" spans="1:8" ht="86.4">
@@ -27285,7 +27243,7 @@
         <v>296</v>
       </c>
       <c r="H125" s="3" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
     </row>
     <row r="126" spans="1:8" ht="28.8">
@@ -27311,7 +27269,7 @@
         <v>298</v>
       </c>
       <c r="H126" s="6" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
     </row>
     <row r="127" spans="1:8" ht="28.8">
@@ -27337,7 +27295,7 @@
         <v>300</v>
       </c>
       <c r="H127" s="8" t="s">
-        <v>703</v>
+        <v>700</v>
       </c>
     </row>
     <row r="128" spans="1:8" ht="28.8">
@@ -27363,7 +27321,7 @@
         <v>302</v>
       </c>
       <c r="H128" s="8" t="s">
-        <v>715</v>
+        <v>711</v>
       </c>
     </row>
     <row r="129" spans="1:8" ht="28.8">
@@ -27389,7 +27347,7 @@
         <v>304</v>
       </c>
       <c r="H129" s="8" t="s">
-        <v>804</v>
+        <v>793</v>
       </c>
     </row>
     <row r="130" spans="1:8" ht="28.8">
@@ -27415,7 +27373,7 @@
         <v>306</v>
       </c>
       <c r="H130" s="8" t="s">
-        <v>805</v>
+        <v>794</v>
       </c>
     </row>
     <row r="131" spans="1:8">
@@ -27467,7 +27425,7 @@
         <v>311</v>
       </c>
       <c r="H132" s="3" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
     </row>
     <row r="133" spans="1:8">
@@ -27493,7 +27451,7 @@
         <v>313</v>
       </c>
       <c r="H133" s="3" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
     </row>
     <row r="134" spans="1:8" ht="28.8">
@@ -27519,7 +27477,7 @@
         <v>316</v>
       </c>
       <c r="H134" s="6" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
     </row>
     <row r="135" spans="1:8" ht="403.2">
@@ -27545,7 +27503,7 @@
         <v>318</v>
       </c>
       <c r="H135" s="3" t="s">
-        <v>727</v>
+        <v>803</v>
       </c>
     </row>
     <row r="136" spans="1:8">
@@ -27571,7 +27529,7 @@
         <v>321</v>
       </c>
       <c r="H136" s="6" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
     </row>
     <row r="137" spans="1:8" ht="43.2">
@@ -27585,7 +27543,7 @@
         <v>1</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>763</v>
+        <v>753</v>
       </c>
       <c r="E137" s="2" t="s">
         <v>11</v>
@@ -27594,13 +27552,13 @@
         <v>12</v>
       </c>
       <c r="G137" s="3" t="s">
-        <v>764</v>
+        <v>754</v>
       </c>
       <c r="H137" s="6" t="s">
-        <v>762</v>
+        <v>752</v>
       </c>
     </row>
-    <row r="138" spans="1:8" ht="100.8">
+    <row r="138" spans="1:8" ht="115.2">
       <c r="A138" s="2" t="s">
         <v>8</v>
       </c>
@@ -27611,7 +27569,7 @@
         <v>2</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>724</v>
+        <v>796</v>
       </c>
       <c r="E138" s="2" t="s">
         <v>11</v>
@@ -27620,24 +27578,24 @@
         <v>12</v>
       </c>
       <c r="G138" s="3" t="s">
-        <v>725</v>
+        <v>797</v>
       </c>
       <c r="H138" s="3" t="s">
-        <v>704</v>
+        <v>798</v>
       </c>
     </row>
     <row r="139" spans="1:8" ht="115.2">
       <c r="A139" s="2" t="s">
-        <v>733</v>
+        <v>725</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>743</v>
+        <v>734</v>
       </c>
       <c r="C139" s="2">
         <v>0</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>744</v>
+        <v>735</v>
       </c>
       <c r="E139" s="2" t="s">
         <v>11</v>
@@ -27646,10 +27604,10 @@
         <v>12</v>
       </c>
       <c r="G139" s="3" t="s">
-        <v>745</v>
+        <v>736</v>
       </c>
       <c r="H139" s="3" t="s">
-        <v>746</v>
+        <v>737</v>
       </c>
     </row>
     <row r="140" spans="1:8" ht="409.6">
@@ -27675,7 +27633,7 @@
         <v>323</v>
       </c>
       <c r="H140" s="3" t="s">
-        <v>755</v>
+        <v>746</v>
       </c>
     </row>
     <row r="141" spans="1:8" ht="28.8">
@@ -27701,7 +27659,7 @@
         <v>326</v>
       </c>
       <c r="H141" s="6" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
     </row>
     <row r="142" spans="1:8">
@@ -27727,7 +27685,7 @@
         <v>329</v>
       </c>
       <c r="H142" s="6" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
     </row>
     <row r="143" spans="1:8" ht="57.6">
@@ -27753,7 +27711,7 @@
         <v>331</v>
       </c>
       <c r="H143" s="6" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
     </row>
     <row r="144" spans="1:8">
@@ -27779,7 +27737,7 @@
         <v>333</v>
       </c>
       <c r="H144" s="6" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
     </row>
     <row r="145" spans="1:8" ht="43.2">
@@ -27805,7 +27763,7 @@
         <v>335</v>
       </c>
       <c r="H145" s="6" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
     </row>
     <row r="146" spans="1:8" ht="86.4">
@@ -27831,7 +27789,7 @@
         <v>337</v>
       </c>
       <c r="H146" s="3" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
     </row>
     <row r="147" spans="1:8" ht="216">
@@ -27857,7 +27815,7 @@
         <v>339</v>
       </c>
       <c r="H147" s="3" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
     </row>
     <row r="148" spans="1:8" ht="86.4">
@@ -27909,7 +27867,7 @@
         <v>345</v>
       </c>
       <c r="H149" s="3" t="s">
-        <v>749</v>
+        <v>740</v>
       </c>
     </row>
     <row r="150" spans="1:8">
@@ -27961,7 +27919,7 @@
         <v>351</v>
       </c>
       <c r="H151" s="3" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
     </row>
     <row r="152" spans="1:8" ht="28.8">
@@ -27987,7 +27945,7 @@
         <v>354</v>
       </c>
       <c r="H152" s="3" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
     </row>
     <row r="153" spans="1:8">
@@ -28013,7 +27971,7 @@
         <v>356</v>
       </c>
       <c r="H153" s="3" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
     </row>
     <row r="154" spans="1:8" ht="129.6">
@@ -28039,7 +27997,7 @@
         <v>359</v>
       </c>
       <c r="H154" s="3" t="s">
-        <v>728</v>
+        <v>721</v>
       </c>
     </row>
     <row r="155" spans="1:8" ht="28.8">
@@ -28117,7 +28075,7 @@
         <v>368</v>
       </c>
       <c r="H157" s="3" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
     </row>
     <row r="158" spans="1:8" ht="28.8">
@@ -28143,7 +28101,7 @@
         <v>371</v>
       </c>
       <c r="H158" s="6" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
     </row>
     <row r="159" spans="1:8" ht="409.6">
@@ -28169,7 +28127,7 @@
         <v>373</v>
       </c>
       <c r="H159" s="3" t="s">
-        <v>705</v>
+        <v>701</v>
       </c>
     </row>
     <row r="160" spans="1:8" ht="43.2">
@@ -28195,7 +28153,7 @@
         <v>376</v>
       </c>
       <c r="H160" s="6" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
     </row>
     <row r="161" spans="1:8" ht="86.4">
@@ -28273,7 +28231,7 @@
         <v>385</v>
       </c>
       <c r="H163" s="6" t="s">
-        <v>706</v>
+        <v>702</v>
       </c>
     </row>
     <row r="164" spans="1:8" ht="100.8">
@@ -28299,7 +28257,7 @@
         <v>388</v>
       </c>
       <c r="H164" s="3" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
     </row>
     <row r="165" spans="1:8" ht="144">
@@ -28325,7 +28283,7 @@
         <v>390</v>
       </c>
       <c r="H165" s="3" t="s">
-        <v>707</v>
+        <v>703</v>
       </c>
     </row>
     <row r="166" spans="1:8" ht="100.8">
@@ -28351,7 +28309,7 @@
         <v>393</v>
       </c>
       <c r="H166" s="3" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
     </row>
     <row r="167" spans="1:8" ht="43.2">
@@ -28377,7 +28335,7 @@
         <v>395</v>
       </c>
       <c r="H167" s="6" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
     </row>
     <row r="168" spans="1:8" ht="115.2">
@@ -28403,7 +28361,7 @@
         <v>398</v>
       </c>
       <c r="H168" s="3" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
     </row>
     <row r="169" spans="1:8" ht="86.4">
@@ -28481,7 +28439,7 @@
         <v>408</v>
       </c>
       <c r="H171" s="3" t="s">
-        <v>708</v>
+        <v>704</v>
       </c>
     </row>
     <row r="172" spans="1:8" ht="57.6">
@@ -28533,7 +28491,7 @@
         <v>413</v>
       </c>
       <c r="H173" s="3" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
     </row>
     <row r="174" spans="1:8" ht="57.6">
@@ -28559,7 +28517,7 @@
         <v>416</v>
       </c>
       <c r="H174" s="6" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
     </row>
     <row r="175" spans="1:8" ht="28.8">
@@ -28634,10 +28592,10 @@
         <v>12</v>
       </c>
       <c r="G177" s="3" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="H177" s="3" t="s">
-        <v>709</v>
+        <v>705</v>
       </c>
     </row>
     <row r="178" spans="1:8" ht="28.8">
@@ -28677,7 +28635,7 @@
         <v>1</v>
       </c>
       <c r="D179" s="2" t="s">
-        <v>759</v>
+        <v>750</v>
       </c>
       <c r="E179" s="2" t="s">
         <v>11</v>
@@ -28686,10 +28644,10 @@
         <v>12</v>
       </c>
       <c r="G179" s="3" t="s">
-        <v>760</v>
+        <v>751</v>
       </c>
       <c r="H179" s="3" t="s">
-        <v>761</v>
+        <v>804</v>
       </c>
     </row>
     <row r="180" spans="1:8" ht="201.6">
@@ -28715,7 +28673,7 @@
         <v>430</v>
       </c>
       <c r="H180" s="3" t="s">
-        <v>737</v>
+        <v>805</v>
       </c>
     </row>
     <row r="181" spans="1:8" ht="86.4">
@@ -28741,7 +28699,7 @@
         <v>433</v>
       </c>
       <c r="H181" s="3" t="s">
-        <v>729</v>
+        <v>806</v>
       </c>
     </row>
     <row r="182" spans="1:8">
@@ -28793,7 +28751,7 @@
         <v>439</v>
       </c>
       <c r="H183" s="6" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
     </row>
     <row r="184" spans="1:8">
@@ -28819,7 +28777,7 @@
         <v>442</v>
       </c>
       <c r="H184" s="6" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
     </row>
     <row r="185" spans="1:8">
@@ -28845,7 +28803,7 @@
         <v>445</v>
       </c>
       <c r="H185" s="6" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
     </row>
     <row r="186" spans="1:8">
@@ -28871,7 +28829,7 @@
         <v>448</v>
       </c>
       <c r="H186" s="6" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
     </row>
     <row r="187" spans="1:8">
@@ -28897,7 +28855,7 @@
         <v>451</v>
       </c>
       <c r="H187" s="6" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
     </row>
     <row r="188" spans="1:8" ht="144">
@@ -28923,7 +28881,7 @@
         <v>454</v>
       </c>
       <c r="H188" s="3" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
     </row>
     <row r="189" spans="1:8" ht="28.8">
@@ -29157,7 +29115,7 @@
         <v>480</v>
       </c>
       <c r="H197" s="6" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
     </row>
     <row r="198" spans="1:8">
@@ -29235,7 +29193,7 @@
         <v>488</v>
       </c>
       <c r="H200" t="s">
-        <v>710</v>
+        <v>706</v>
       </c>
     </row>
     <row r="201" spans="1:8">
@@ -29261,7 +29219,7 @@
         <v>490</v>
       </c>
       <c r="H201" s="6" t="s">
-        <v>711</v>
+        <v>707</v>
       </c>
     </row>
     <row r="202" spans="1:8" ht="100.8">
@@ -29287,7 +29245,7 @@
         <v>492</v>
       </c>
       <c r="H202" s="3" t="s">
-        <v>730</v>
+        <v>722</v>
       </c>
     </row>
     <row r="203" spans="1:8" ht="158.4">
@@ -29313,7 +29271,7 @@
         <v>494</v>
       </c>
       <c r="H203" s="3" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
     </row>
     <row r="204" spans="1:8" ht="43.2">
@@ -29339,7 +29297,7 @@
         <v>496</v>
       </c>
       <c r="H204" s="3" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
     </row>
     <row r="205" spans="1:8" ht="100.8">
@@ -29365,7 +29323,7 @@
         <v>498</v>
       </c>
       <c r="H205" s="3" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
     </row>
     <row r="206" spans="1:8" ht="43.2">
@@ -29391,7 +29349,7 @@
         <v>500</v>
       </c>
       <c r="H206" s="3" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
     </row>
     <row r="207" spans="1:8" ht="100.8">
@@ -29417,7 +29375,7 @@
         <v>502</v>
       </c>
       <c r="H207" s="3" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
     </row>
     <row r="208" spans="1:8" ht="100.8">
@@ -29443,7 +29401,7 @@
         <v>504</v>
       </c>
       <c r="H208" s="3" t="s">
-        <v>712</v>
+        <v>708</v>
       </c>
     </row>
     <row r="209" spans="1:9" ht="115.2">
@@ -29469,7 +29427,7 @@
         <v>506</v>
       </c>
       <c r="H209" s="3" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="210" spans="1:9" ht="158.4">
@@ -29495,7 +29453,7 @@
         <v>508</v>
       </c>
       <c r="H210" s="3" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
     </row>
     <row r="211" spans="1:9" ht="172.8">
@@ -29521,7 +29479,7 @@
         <v>510</v>
       </c>
       <c r="H211" s="3" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="212" spans="1:9" ht="115.2">
@@ -29547,7 +29505,7 @@
         <v>512</v>
       </c>
       <c r="H212" s="3" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
     </row>
     <row r="213" spans="1:9" ht="158.4">
@@ -29570,10 +29528,10 @@
         <v>12</v>
       </c>
       <c r="G213" s="3" t="s">
-        <v>731</v>
+        <v>723</v>
       </c>
       <c r="H213" s="3" t="s">
-        <v>732</v>
+        <v>724</v>
       </c>
     </row>
     <row r="214" spans="1:9" ht="158.4">
@@ -29599,7 +29557,7 @@
         <v>515</v>
       </c>
       <c r="H214" s="3" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
     </row>
     <row r="215" spans="1:9" ht="187.2">
@@ -29613,7 +29571,7 @@
         <v>16</v>
       </c>
       <c r="D215" s="2" t="s">
-        <v>790</v>
+        <v>780</v>
       </c>
       <c r="E215" s="2" t="s">
         <v>11</v>
@@ -29622,10 +29580,10 @@
         <v>12</v>
       </c>
       <c r="G215" s="3" t="s">
-        <v>792</v>
+        <v>782</v>
       </c>
       <c r="H215" s="3" t="s">
-        <v>793</v>
+        <v>783</v>
       </c>
     </row>
     <row r="216" spans="1:9" ht="187.2">
@@ -29639,7 +29597,7 @@
         <v>17</v>
       </c>
       <c r="D216" s="2" t="s">
-        <v>791</v>
+        <v>781</v>
       </c>
       <c r="E216" s="2" t="s">
         <v>11</v>
@@ -29648,10 +29606,10 @@
         <v>12</v>
       </c>
       <c r="G216" s="3" t="s">
-        <v>794</v>
+        <v>784</v>
       </c>
       <c r="H216" s="3" t="s">
-        <v>795</v>
+        <v>785</v>
       </c>
     </row>
     <row r="217" spans="1:9" ht="100.8">
@@ -29665,7 +29623,7 @@
         <v>18</v>
       </c>
       <c r="D217" s="2" t="s">
-        <v>784</v>
+        <v>774</v>
       </c>
       <c r="E217" s="2" t="s">
         <v>11</v>
@@ -29674,10 +29632,10 @@
         <v>12</v>
       </c>
       <c r="G217" s="3" t="s">
-        <v>785</v>
+        <v>775</v>
       </c>
       <c r="H217" s="3" t="s">
-        <v>788</v>
+        <v>778</v>
       </c>
     </row>
     <row r="218" spans="1:9" ht="100.8">
@@ -29691,7 +29649,7 @@
         <v>19</v>
       </c>
       <c r="D218" s="2" t="s">
-        <v>786</v>
+        <v>776</v>
       </c>
       <c r="E218" s="2" t="s">
         <v>11</v>
@@ -29700,10 +29658,10 @@
         <v>12</v>
       </c>
       <c r="G218" s="3" t="s">
-        <v>787</v>
+        <v>777</v>
       </c>
       <c r="H218" s="3" t="s">
-        <v>789</v>
+        <v>779</v>
       </c>
     </row>
     <row r="219" spans="1:9" ht="43.2">
@@ -29729,7 +29687,7 @@
         <v>517</v>
       </c>
       <c r="H219" s="3" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
     </row>
     <row r="220" spans="1:9" ht="409.6">
@@ -29743,7 +29701,7 @@
         <v>21</v>
       </c>
       <c r="D220" s="2" t="s">
-        <v>756</v>
+        <v>747</v>
       </c>
       <c r="E220" s="2" t="s">
         <v>11</v>
@@ -29752,14 +29710,14 @@
         <v>12</v>
       </c>
       <c r="G220" s="3" t="s">
-        <v>757</v>
+        <v>748</v>
       </c>
       <c r="H220" s="3" t="s">
-        <v>758</v>
+        <v>749</v>
       </c>
       <c r="I220" s="3"/>
     </row>
-    <row r="221" spans="1:9" ht="115.2">
+    <row r="221" spans="1:9" ht="129.6">
       <c r="A221" s="2" t="s">
         <v>8</v>
       </c>
@@ -29770,7 +29728,7 @@
         <v>22</v>
       </c>
       <c r="D221" s="2" t="s">
-        <v>518</v>
+        <v>799</v>
       </c>
       <c r="E221" s="2" t="s">
         <v>11</v>
@@ -29779,10 +29737,10 @@
         <v>12</v>
       </c>
       <c r="G221" s="3" t="s">
-        <v>519</v>
+        <v>800</v>
       </c>
       <c r="H221" s="3" t="s">
-        <v>690</v>
+        <v>801</v>
       </c>
     </row>
     <row r="222" spans="1:9" ht="43.2">
@@ -29796,7 +29754,7 @@
         <v>23</v>
       </c>
       <c r="D222" s="2" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="E222" s="2" t="s">
         <v>11</v>
@@ -29805,10 +29763,10 @@
         <v>12</v>
       </c>
       <c r="G222" s="3" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="H222" s="3" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
     </row>
     <row r="223" spans="1:9" ht="86.4">
@@ -29822,7 +29780,7 @@
         <v>24</v>
       </c>
       <c r="D223" s="2" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="E223" s="2" t="s">
         <v>11</v>
@@ -29831,10 +29789,10 @@
         <v>12</v>
       </c>
       <c r="G223" s="3" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="H223" s="3" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
     </row>
     <row r="224" spans="1:9" ht="115.2">
@@ -29848,7 +29806,7 @@
         <v>25</v>
       </c>
       <c r="D224" s="2" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="E224" s="2" t="s">
         <v>11</v>
@@ -29857,10 +29815,10 @@
         <v>12</v>
       </c>
       <c r="G224" s="3" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="H224" s="3" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
     </row>
     <row r="225" spans="1:8" ht="43.2">
@@ -29874,7 +29832,7 @@
         <v>26</v>
       </c>
       <c r="D225" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="E225" s="2" t="s">
         <v>11</v>
@@ -29883,10 +29841,10 @@
         <v>12</v>
       </c>
       <c r="G225" s="3" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="H225" s="3" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
     </row>
     <row r="226" spans="1:8" ht="100.8">
@@ -29900,7 +29858,7 @@
         <v>27</v>
       </c>
       <c r="D226" s="2" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="E226" s="2" t="s">
         <v>11</v>
@@ -29909,10 +29867,10 @@
         <v>12</v>
       </c>
       <c r="G226" s="3" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="H226" s="3" t="s">
-        <v>713</v>
+        <v>709</v>
       </c>
     </row>
     <row r="227" spans="1:8" ht="43.2">
@@ -29926,7 +29884,7 @@
         <v>28</v>
       </c>
       <c r="D227" s="2" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="E227" s="2" t="s">
         <v>11</v>
@@ -29935,10 +29893,10 @@
         <v>12</v>
       </c>
       <c r="G227" s="3" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="H227" s="3" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
     </row>
     <row r="228" spans="1:8" ht="43.2">
@@ -29952,7 +29910,7 @@
         <v>29</v>
       </c>
       <c r="D228" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="E228" s="2" t="s">
         <v>11</v>
@@ -29961,10 +29919,10 @@
         <v>12</v>
       </c>
       <c r="G228" s="3" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="H228" s="3" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
     </row>
     <row r="229" spans="1:8" ht="100.8">
@@ -29978,7 +29936,7 @@
         <v>30</v>
       </c>
       <c r="D229" s="2" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="E229" s="2" t="s">
         <v>11</v>
@@ -29987,10 +29945,10 @@
         <v>12</v>
       </c>
       <c r="G229" s="3" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="H229" s="3" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
     </row>
     <row r="230" spans="1:8" ht="28.8">
@@ -29998,13 +29956,13 @@
         <v>8</v>
       </c>
       <c r="B230" s="2" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="C230" s="2">
         <v>0</v>
       </c>
       <c r="D230" s="2" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="E230" s="2" t="s">
         <v>11</v>
@@ -30013,10 +29971,10 @@
         <v>12</v>
       </c>
       <c r="G230" s="3" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="H230" s="6" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
     </row>
     <row r="231" spans="1:8" ht="28.8">
@@ -30024,13 +29982,13 @@
         <v>8</v>
       </c>
       <c r="B231" s="2" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="C231" s="2">
         <v>0</v>
       </c>
       <c r="D231" s="2" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="E231" s="2" t="s">
         <v>11</v>
@@ -30039,10 +29997,10 @@
         <v>12</v>
       </c>
       <c r="G231" s="3" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="H231" s="3" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
     </row>
     <row r="232" spans="1:8" ht="43.2">
@@ -30050,13 +30008,13 @@
         <v>8</v>
       </c>
       <c r="B232" s="2" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="C232" s="2">
         <v>1</v>
       </c>
       <c r="D232" s="2" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="E232" s="2" t="s">
         <v>11</v>
@@ -30065,10 +30023,10 @@
         <v>12</v>
       </c>
       <c r="G232" s="3" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="H232" s="3" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
     </row>
     <row r="233" spans="1:8" ht="100.8">
@@ -30076,13 +30034,13 @@
         <v>8</v>
       </c>
       <c r="B233" s="2" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="C233" s="2">
         <v>2</v>
       </c>
       <c r="D233" s="2" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="E233" s="2" t="s">
         <v>11</v>
@@ -30091,10 +30049,10 @@
         <v>12</v>
       </c>
       <c r="G233" s="3" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="H233" s="3" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
     </row>
     <row r="234" spans="1:8" ht="43.2">
@@ -30102,13 +30060,13 @@
         <v>8</v>
       </c>
       <c r="B234" s="2" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="C234" s="2">
         <v>3</v>
       </c>
       <c r="D234" s="2" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="E234" s="2" t="s">
         <v>11</v>
@@ -30117,10 +30075,10 @@
         <v>12</v>
       </c>
       <c r="G234" s="3" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="H234" s="3" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
     </row>
     <row r="235" spans="1:8">
@@ -30128,13 +30086,13 @@
         <v>8</v>
       </c>
       <c r="B235" s="2" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="C235" s="2">
         <v>0</v>
       </c>
       <c r="D235" s="2" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="E235" s="2" t="s">
         <v>11</v>
@@ -30143,10 +30101,10 @@
         <v>12</v>
       </c>
       <c r="G235" s="3" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="H235" s="6" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
     </row>
     <row r="236" spans="1:8">
@@ -30154,13 +30112,13 @@
         <v>8</v>
       </c>
       <c r="B236" s="2" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="C236" s="2">
         <v>0</v>
       </c>
       <c r="D236" s="2" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="E236" s="2" t="s">
         <v>11</v>
@@ -30169,10 +30127,10 @@
         <v>12</v>
       </c>
       <c r="G236" s="3" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="H236" s="6" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
     </row>
     <row r="237" spans="1:8" ht="28.8">
@@ -30180,13 +30138,13 @@
         <v>8</v>
       </c>
       <c r="B237" s="2" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="C237" s="2">
         <v>1</v>
       </c>
       <c r="D237" s="2" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="E237" s="2" t="s">
         <v>11</v>
@@ -30195,10 +30153,10 @@
         <v>12</v>
       </c>
       <c r="G237" s="3" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="H237" s="6" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
     </row>
     <row r="238" spans="1:8">
@@ -30206,13 +30164,13 @@
         <v>8</v>
       </c>
       <c r="B238" s="2" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="C238" s="2">
         <v>0</v>
       </c>
       <c r="D238" s="2" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="E238" s="2" t="s">
         <v>11</v>
@@ -30221,10 +30179,10 @@
         <v>12</v>
       </c>
       <c r="G238" s="3" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="H238" s="6" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
     </row>
     <row r="239" spans="1:8" ht="28.8">
@@ -30232,13 +30190,13 @@
         <v>8</v>
       </c>
       <c r="B239" s="2" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="C239" s="2">
         <v>1</v>
       </c>
       <c r="D239" s="2" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="E239" s="2" t="s">
         <v>11</v>
@@ -30247,10 +30205,10 @@
         <v>12</v>
       </c>
       <c r="G239" s="3" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="H239" s="4" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
     </row>
     <row r="240" spans="1:8">
@@ -30258,13 +30216,13 @@
         <v>8</v>
       </c>
       <c r="B240" s="2" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="C240" s="2">
         <v>0</v>
       </c>
       <c r="D240" s="2" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="E240" s="2" t="s">
         <v>11</v>
@@ -30273,7 +30231,7 @@
         <v>12</v>
       </c>
       <c r="G240" s="3" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="H240" s="4" t="s">
         <v>23</v>
@@ -30284,13 +30242,13 @@
         <v>8</v>
       </c>
       <c r="B241" s="2" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="C241" s="2">
         <v>1</v>
       </c>
       <c r="D241" s="2" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="E241" s="2" t="s">
         <v>11</v>
@@ -30299,10 +30257,10 @@
         <v>12</v>
       </c>
       <c r="G241" s="3" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="H241" s="4" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
     </row>
     <row r="242" spans="1:8">
@@ -30310,13 +30268,13 @@
         <v>8</v>
       </c>
       <c r="B242" s="2" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="C242" s="2">
         <v>0</v>
       </c>
       <c r="D242" s="2" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="E242" s="2" t="s">
         <v>11</v>
@@ -30325,24 +30283,24 @@
         <v>12</v>
       </c>
       <c r="G242" s="3" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="H242" s="4" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
     </row>
     <row r="243" spans="1:8">
       <c r="A243" t="s">
-        <v>733</v>
+        <v>725</v>
       </c>
       <c r="B243" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="C243">
         <v>1</v>
       </c>
       <c r="D243" t="s">
-        <v>734</v>
+        <v>726</v>
       </c>
       <c r="E243" t="s">
         <v>11</v>
@@ -30351,10 +30309,10 @@
         <v>12</v>
       </c>
       <c r="G243" t="s">
-        <v>735</v>
+        <v>727</v>
       </c>
       <c r="H243" s="4" t="s">
-        <v>736</v>
+        <v>728</v>
       </c>
     </row>
     <row r="244" spans="1:8">

</xml_diff>